<commit_message>
feat: implement ATT V1.1 runtime
</commit_message>
<xml_diff>
--- a/testcase/payment_regression.xlsx
+++ b/testcase/payment_regression.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TestCases" sheetId="1" r:id="Rcab596a42a1c4128"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Config" sheetId="2" r:id="Ra92e4df4ec6149b9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="3" r:id="Radbae07e9d444f80"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TestCases" sheetId="1" r:id="R1c901ee28e4c420c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Config" sheetId="2" r:id="R2bdb8b288b344200"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="3" r:id="Raf2e949e057f42a3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -279,27 +279,27 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="32" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="24" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="18" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="18" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="18" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="18" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="18" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="28" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="18" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="44" hidden="0" customWidth="1"/>
-    <x:col min="17" max="17" width="48" hidden="0" customWidth="1"/>
-    <x:col min="18" max="18" width="48" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="6.21999979019165" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="35.220001220703125" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="22.559999465942383" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="8" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="17.559999465942383" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="20" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="18.889999389648438" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="17.110000610351562" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="10.890000343322754" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="11.4399995803833" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="8.220000267028809" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="7.110000133514404" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="23.889999389648438" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="18.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="20.889999389648438" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="21.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="41.220001220703125" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="17.440000534057617" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1">
+    <x:row r="1" ht="15" hidden="0" customHeight="1">
       <x:c r="A1" s="5" t="str">
         <x:v>Case ID</x:v>
       </x:c>
@@ -355,15 +355,15 @@
         <x:v>Ignored Helper Column</x:v>
       </x:c>
     </x:row>
-    <x:row r="2">
+    <x:row r="2" ht="79.19999694824219" hidden="0" customHeight="1">
       <x:c r="A2" s="6" t="str">
         <x:v>TC001</x:v>
       </x:c>
       <x:c r="B2" s="6" t="str">
-        <x:v>Payment transfer success</x:v>
+        <x:v>ATM HKD transfer success</x:v>
       </x:c>
       <x:c r="C2" s="6" t="str">
-        <x:v>smoke,regression</x:v>
+        <x:v>smoke,regression,atm</x:v>
       </x:c>
       <x:c r="D2" s="6" t="str">
         <x:v>PAYMENT</x:v>
@@ -393,7 +393,8 @@
         <x:v>HKD</x:v>
       </x:c>
       <x:c r="M2" s="6" t="str">
-        <x:v>channel: ATM</x:v>
+        <x:v>channel: ATM
+priority: NORMAL</x:v>
       </x:c>
       <x:c r="N2" s="6" t="str">
         <x:v>PAYMENT_POSTCHECK</x:v>
@@ -410,21 +411,21 @@
 Keyword2: POSTED</x:v>
       </x:c>
       <x:c r="Q2" s="6" t="str">
-        <x:v>Happy path. Last column is intentionally not configured and should be ignored.</x:v>
+        <x:v>Happy path for ATM HKD transfer.</x:v>
       </x:c>
       <x:c r="R2" s="6" t="str">
         <x:v>ATT should ignore this</x:v>
       </x:c>
     </x:row>
-    <x:row r="3">
+    <x:row r="3" ht="79.19999694824219" hidden="0" customHeight="1">
       <x:c r="A3" s="6" t="str">
         <x:v>TC002</x:v>
       </x:c>
       <x:c r="B3" s="6" t="str">
-        <x:v>Mobile payment transfer success</x:v>
+        <x:v>Mobile HKD small amount success</x:v>
       </x:c>
       <x:c r="C3" s="6" t="str">
-        <x:v>smoke,mobile</x:v>
+        <x:v>smoke,mobile,low-value</x:v>
       </x:c>
       <x:c r="D3" s="6" t="str">
         <x:v>PAYMENT</x:v>
@@ -454,7 +455,8 @@
         <x:v>HKD</x:v>
       </x:c>
       <x:c r="M3" s="6" t="str">
-        <x:v>channel: MOBILE</x:v>
+        <x:v>channel: MOBILE
+priority: NORMAL</x:v>
       </x:c>
       <x:c r="N3" s="6" t="str">
         <x:v>PAYMENT_POSTCHECK</x:v>
@@ -471,9 +473,1125 @@
 Keyword2: POSTED</x:v>
       </x:c>
       <x:c r="Q3" s="6" t="str">
-        <x:v>Covers configured fields with a mobile channel.</x:v>
+        <x:v>Minimum positive amount through mobile channel.</x:v>
       </x:c>
       <x:c r="R3" s="6" t="str">
+        <x:v>ATT should ignore this</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A4" s="6" t="str">
+        <x:v>TC003</x:v>
+      </x:c>
+      <x:c r="B4" s="6" t="str">
+        <x:v>Internet banking HKD large amount success</x:v>
+      </x:c>
+      <x:c r="C4" s="6" t="str">
+        <x:v>regression,web,high-value</x:v>
+      </x:c>
+      <x:c r="D4" s="6" t="str">
+        <x:v>PAYMENT</x:v>
+      </x:c>
+      <x:c r="E4" s="6" t="str">
+        <x:v>PAYMENT_PRECHECK</x:v>
+      </x:c>
+      <x:c r="F4" s="6" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="G4" s="6" t="str">
+        <x:v>minAccountRows: 1</x:v>
+      </x:c>
+      <x:c r="H4" s="6" t="str">
+        <x:v>PAYMENT_TRANSFER</x:v>
+      </x:c>
+      <x:c r="I4" s="6" t="str">
+        <x:v>111113</x:v>
+      </x:c>
+      <x:c r="J4" s="6" t="str">
+        <x:v>222224</x:v>
+      </x:c>
+      <x:c r="K4" s="6" t="str">
+        <x:v>999999.99</x:v>
+      </x:c>
+      <x:c r="L4" s="6" t="str">
+        <x:v>HKD</x:v>
+      </x:c>
+      <x:c r="M4" s="6" t="str">
+        <x:v>channel: WEB
+priority: HIGH</x:v>
+      </x:c>
+      <x:c r="N4" s="6" t="str">
+        <x:v>PAYMENT_POSTCHECK</x:v>
+      </x:c>
+      <x:c r="O4" s="6" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="P4" s="6" t="str">
+        <x:v>expectedStatus: SUCCESS
+expectedRejectCode: '0000'
+effectedRows: 1
+status: POSTED
+Keyword1: PAYMENT
+Keyword2: POSTED</x:v>
+      </x:c>
+      <x:c r="Q4" s="6" t="str">
+        <x:v>Large amount with high priority marker.</x:v>
+      </x:c>
+      <x:c r="R4" s="6" t="str">
+        <x:v>ATT should ignore this</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A5" s="6" t="str">
+        <x:v>TC004</x:v>
+      </x:c>
+      <x:c r="B5" s="6" t="str">
+        <x:v>Branch assisted HKD round amount success</x:v>
+      </x:c>
+      <x:c r="C5" s="6" t="str">
+        <x:v>regression,branch</x:v>
+      </x:c>
+      <x:c r="D5" s="6" t="str">
+        <x:v>PAYMENT</x:v>
+      </x:c>
+      <x:c r="E5" s="6" t="str">
+        <x:v>PAYMENT_PRECHECK</x:v>
+      </x:c>
+      <x:c r="F5" s="6" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="G5" s="6" t="str">
+        <x:v>minAccountRows: 1</x:v>
+      </x:c>
+      <x:c r="H5" s="6" t="str">
+        <x:v>PAYMENT_TRANSFER</x:v>
+      </x:c>
+      <x:c r="I5" s="6" t="str">
+        <x:v>111114</x:v>
+      </x:c>
+      <x:c r="J5" s="6" t="str">
+        <x:v>222225</x:v>
+      </x:c>
+      <x:c r="K5" s="6" t="str">
+        <x:v>5000</x:v>
+      </x:c>
+      <x:c r="L5" s="6" t="str">
+        <x:v>HKD</x:v>
+      </x:c>
+      <x:c r="M5" s="6" t="str">
+        <x:v>channel: BRANCH
+priority: NORMAL</x:v>
+      </x:c>
+      <x:c r="N5" s="6" t="str">
+        <x:v>PAYMENT_POSTCHECK</x:v>
+      </x:c>
+      <x:c r="O5" s="6" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="P5" s="6" t="str">
+        <x:v>expectedStatus: SUCCESS
+expectedRejectCode: '0000'
+effectedRows: 1
+status: POSTED
+Keyword1: PAYMENT
+Keyword2: POSTED</x:v>
+      </x:c>
+      <x:c r="Q5" s="6" t="str">
+        <x:v>Branch-assisted transfer.</x:v>
+      </x:c>
+      <x:c r="R5" s="6" t="str">
+        <x:v>ATT should ignore this</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A6" s="6" t="str">
+        <x:v>TC005</x:v>
+      </x:c>
+      <x:c r="B6" s="6" t="str">
+        <x:v>Corporate payroll transfer success</x:v>
+      </x:c>
+      <x:c r="C6" s="6" t="str">
+        <x:v>regression,corporate,payroll</x:v>
+      </x:c>
+      <x:c r="D6" s="6" t="str">
+        <x:v>PAYMENT</x:v>
+      </x:c>
+      <x:c r="E6" s="6" t="str">
+        <x:v>PAYMENT_PRECHECK</x:v>
+      </x:c>
+      <x:c r="F6" s="6" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="G6" s="6" t="str">
+        <x:v>minAccountRows: 1</x:v>
+      </x:c>
+      <x:c r="H6" s="6" t="str">
+        <x:v>PAYMENT_TRANSFER</x:v>
+      </x:c>
+      <x:c r="I6" s="6" t="str">
+        <x:v>311115</x:v>
+      </x:c>
+      <x:c r="J6" s="6" t="str">
+        <x:v>422226</x:v>
+      </x:c>
+      <x:c r="K6" s="6" t="str">
+        <x:v>88888.88</x:v>
+      </x:c>
+      <x:c r="L6" s="6" t="str">
+        <x:v>HKD</x:v>
+      </x:c>
+      <x:c r="M6" s="6" t="str">
+        <x:v>channel: HOST
+purpose: PAYROLL</x:v>
+      </x:c>
+      <x:c r="N6" s="6" t="str">
+        <x:v>PAYMENT_POSTCHECK</x:v>
+      </x:c>
+      <x:c r="O6" s="6" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="P6" s="6" t="str">
+        <x:v>expectedStatus: SUCCESS
+expectedRejectCode: '0000'
+effectedRows: 1
+status: POSTED
+Keyword1: PAYMENT
+Keyword2: POSTED</x:v>
+      </x:c>
+      <x:c r="Q6" s="6" t="str">
+        <x:v>Corporate payroll-like payment.</x:v>
+      </x:c>
+      <x:c r="R6" s="6" t="str">
+        <x:v>ATT should ignore this</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A7" s="6" t="str">
+        <x:v>TC006</x:v>
+      </x:c>
+      <x:c r="B7" s="6" t="str">
+        <x:v>Treasury USD transfer success</x:v>
+      </x:c>
+      <x:c r="C7" s="6" t="str">
+        <x:v>regression,fx,usd</x:v>
+      </x:c>
+      <x:c r="D7" s="6" t="str">
+        <x:v>PAYMENT</x:v>
+      </x:c>
+      <x:c r="E7" s="6" t="str">
+        <x:v>PAYMENT_PRECHECK</x:v>
+      </x:c>
+      <x:c r="F7" s="6" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="G7" s="6" t="str">
+        <x:v>minAccountRows: 1</x:v>
+      </x:c>
+      <x:c r="H7" s="6" t="str">
+        <x:v>PAYMENT_TRANSFER</x:v>
+      </x:c>
+      <x:c r="I7" s="6" t="str">
+        <x:v>511116</x:v>
+      </x:c>
+      <x:c r="J7" s="6" t="str">
+        <x:v>622227</x:v>
+      </x:c>
+      <x:c r="K7" s="6" t="str">
+        <x:v>1234.56</x:v>
+      </x:c>
+      <x:c r="L7" s="6" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="M7" s="6" t="str">
+        <x:v>channel: WEB
+fxRequired: true</x:v>
+      </x:c>
+      <x:c r="N7" s="6" t="str">
+        <x:v>PAYMENT_POSTCHECK</x:v>
+      </x:c>
+      <x:c r="O7" s="6" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="P7" s="6" t="str">
+        <x:v>expectedStatus: SUCCESS
+expectedRejectCode: '0000'
+effectedRows: 1
+status: POSTED
+Keyword1: PAYMENT
+Keyword2: POSTED</x:v>
+      </x:c>
+      <x:c r="Q7" s="6" t="str">
+        <x:v>USD transfer with FX flag.</x:v>
+      </x:c>
+      <x:c r="R7" s="6" t="str">
+        <x:v>ATT should ignore this</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A8" s="6" t="str">
+        <x:v>TC007</x:v>
+      </x:c>
+      <x:c r="B8" s="6" t="str">
+        <x:v>EUR remittance style transfer success</x:v>
+      </x:c>
+      <x:c r="C8" s="6" t="str">
+        <x:v>regression,fx,eur</x:v>
+      </x:c>
+      <x:c r="D8" s="6" t="str">
+        <x:v>PAYMENT</x:v>
+      </x:c>
+      <x:c r="E8" s="6" t="str">
+        <x:v>PAYMENT_PRECHECK</x:v>
+      </x:c>
+      <x:c r="F8" s="6" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="G8" s="6" t="str">
+        <x:v>minAccountRows: 1</x:v>
+      </x:c>
+      <x:c r="H8" s="6" t="str">
+        <x:v>PAYMENT_TRANSFER</x:v>
+      </x:c>
+      <x:c r="I8" s="6" t="str">
+        <x:v>511117</x:v>
+      </x:c>
+      <x:c r="J8" s="6" t="str">
+        <x:v>622228</x:v>
+      </x:c>
+      <x:c r="K8" s="6" t="str">
+        <x:v>789.01</x:v>
+      </x:c>
+      <x:c r="L8" s="6" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="M8" s="6" t="str">
+        <x:v>channel: WEB
+fxRequired: true</x:v>
+      </x:c>
+      <x:c r="N8" s="6" t="str">
+        <x:v>PAYMENT_POSTCHECK</x:v>
+      </x:c>
+      <x:c r="O8" s="6" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="P8" s="6" t="str">
+        <x:v>expectedStatus: SUCCESS
+expectedRejectCode: '0000'
+effectedRows: 1
+status: POSTED
+Keyword1: PAYMENT
+Keyword2: POSTED</x:v>
+      </x:c>
+      <x:c r="Q8" s="6" t="str">
+        <x:v>EUR payment scenario.</x:v>
+      </x:c>
+      <x:c r="R8" s="6" t="str">
+        <x:v>ATT should ignore this</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A9" s="6" t="str">
+        <x:v>TC008</x:v>
+      </x:c>
+      <x:c r="B9" s="6" t="str">
+        <x:v>CNY cross-border transfer success</x:v>
+      </x:c>
+      <x:c r="C9" s="6" t="str">
+        <x:v>regression,fx,cny,cross-border</x:v>
+      </x:c>
+      <x:c r="D9" s="6" t="str">
+        <x:v>PAYMENT</x:v>
+      </x:c>
+      <x:c r="E9" s="6" t="str">
+        <x:v>PAYMENT_PRECHECK</x:v>
+      </x:c>
+      <x:c r="F9" s="6" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="G9" s="6" t="str">
+        <x:v>minAccountRows: 1</x:v>
+      </x:c>
+      <x:c r="H9" s="6" t="str">
+        <x:v>PAYMENT_TRANSFER</x:v>
+      </x:c>
+      <x:c r="I9" s="6" t="str">
+        <x:v>511118</x:v>
+      </x:c>
+      <x:c r="J9" s="6" t="str">
+        <x:v>622229</x:v>
+      </x:c>
+      <x:c r="K9" s="6" t="str">
+        <x:v>3000</x:v>
+      </x:c>
+      <x:c r="L9" s="6" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="M9" s="6" t="str">
+        <x:v>channel: MOBILE
+crossBorder: true</x:v>
+      </x:c>
+      <x:c r="N9" s="6" t="str">
+        <x:v>PAYMENT_POSTCHECK</x:v>
+      </x:c>
+      <x:c r="O9" s="6" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="P9" s="6" t="str">
+        <x:v>expectedStatus: SUCCESS
+expectedRejectCode: '0000'
+effectedRows: 1
+status: POSTED
+Keyword1: PAYMENT
+Keyword2: POSTED</x:v>
+      </x:c>
+      <x:c r="Q9" s="6" t="str">
+        <x:v>CNY cross-border style payment.</x:v>
+      </x:c>
+      <x:c r="R9" s="6" t="str">
+        <x:v>ATT should ignore this</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A10" s="6" t="str">
+        <x:v>TC009</x:v>
+      </x:c>
+      <x:c r="B10" s="6" t="str">
+        <x:v>Same customer own-account transfer success</x:v>
+      </x:c>
+      <x:c r="C10" s="6" t="str">
+        <x:v>regression,own-account</x:v>
+      </x:c>
+      <x:c r="D10" s="6" t="str">
+        <x:v>PAYMENT</x:v>
+      </x:c>
+      <x:c r="E10" s="6" t="str">
+        <x:v>PAYMENT_PRECHECK</x:v>
+      </x:c>
+      <x:c r="F10" s="6" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="G10" s="6" t="str">
+        <x:v>minAccountRows: 1</x:v>
+      </x:c>
+      <x:c r="H10" s="6" t="str">
+        <x:v>PAYMENT_TRANSFER</x:v>
+      </x:c>
+      <x:c r="I10" s="6" t="str">
+        <x:v>711119</x:v>
+      </x:c>
+      <x:c r="J10" s="6" t="str">
+        <x:v>711120</x:v>
+      </x:c>
+      <x:c r="K10" s="6" t="str">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="L10" s="6" t="str">
+        <x:v>HKD</x:v>
+      </x:c>
+      <x:c r="M10" s="6" t="str">
+        <x:v>channel: MOBILE
+relationship: OWN_ACCOUNT</x:v>
+      </x:c>
+      <x:c r="N10" s="6" t="str">
+        <x:v>PAYMENT_POSTCHECK</x:v>
+      </x:c>
+      <x:c r="O10" s="6" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="P10" s="6" t="str">
+        <x:v>expectedStatus: SUCCESS
+expectedRejectCode: '0000'
+effectedRows: 1
+status: POSTED
+Keyword1: PAYMENT
+Keyword2: POSTED</x:v>
+      </x:c>
+      <x:c r="Q10" s="6" t="str">
+        <x:v>Own-account movement.</x:v>
+      </x:c>
+      <x:c r="R10" s="6" t="str">
+        <x:v>ATT should ignore this</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A11" s="6" t="str">
+        <x:v>TC010</x:v>
+      </x:c>
+      <x:c r="B11" s="6" t="str">
+        <x:v>Third-party local transfer success</x:v>
+      </x:c>
+      <x:c r="C11" s="6" t="str">
+        <x:v>regression,third-party</x:v>
+      </x:c>
+      <x:c r="D11" s="6" t="str">
+        <x:v>PAYMENT</x:v>
+      </x:c>
+      <x:c r="E11" s="6" t="str">
+        <x:v>PAYMENT_PRECHECK</x:v>
+      </x:c>
+      <x:c r="F11" s="6" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="G11" s="6" t="str">
+        <x:v>minAccountRows: 1</x:v>
+      </x:c>
+      <x:c r="H11" s="6" t="str">
+        <x:v>PAYMENT_TRANSFER</x:v>
+      </x:c>
+      <x:c r="I11" s="6" t="str">
+        <x:v>711121</x:v>
+      </x:c>
+      <x:c r="J11" s="6" t="str">
+        <x:v>822230</x:v>
+      </x:c>
+      <x:c r="K11" s="6" t="str">
+        <x:v>750</x:v>
+      </x:c>
+      <x:c r="L11" s="6" t="str">
+        <x:v>HKD</x:v>
+      </x:c>
+      <x:c r="M11" s="6" t="str">
+        <x:v>channel: WEB
+relationship: THIRD_PARTY</x:v>
+      </x:c>
+      <x:c r="N11" s="6" t="str">
+        <x:v>PAYMENT_POSTCHECK</x:v>
+      </x:c>
+      <x:c r="O11" s="6" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="P11" s="6" t="str">
+        <x:v>expectedStatus: SUCCESS
+expectedRejectCode: '0000'
+effectedRows: 1
+status: POSTED
+Keyword1: PAYMENT
+Keyword2: POSTED</x:v>
+      </x:c>
+      <x:c r="Q11" s="6" t="str">
+        <x:v>Third-party local transfer.</x:v>
+      </x:c>
+      <x:c r="R11" s="6" t="str">
+        <x:v>ATT should ignore this</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A12" s="6" t="str">
+        <x:v>TC011</x:v>
+      </x:c>
+      <x:c r="B12" s="6" t="str">
+        <x:v>Future-dated transfer success</x:v>
+      </x:c>
+      <x:c r="C12" s="6" t="str">
+        <x:v>regression,future-dated</x:v>
+      </x:c>
+      <x:c r="D12" s="6" t="str">
+        <x:v>PAYMENT</x:v>
+      </x:c>
+      <x:c r="E12" s="6" t="str">
+        <x:v>PAYMENT_PRECHECK</x:v>
+      </x:c>
+      <x:c r="F12" s="6" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="G12" s="6" t="str">
+        <x:v>minAccountRows: 1</x:v>
+      </x:c>
+      <x:c r="H12" s="6" t="str">
+        <x:v>PAYMENT_TRANSFER</x:v>
+      </x:c>
+      <x:c r="I12" s="6" t="str">
+        <x:v>811122</x:v>
+      </x:c>
+      <x:c r="J12" s="6" t="str">
+        <x:v>922231</x:v>
+      </x:c>
+      <x:c r="K12" s="6" t="str">
+        <x:v>1200</x:v>
+      </x:c>
+      <x:c r="L12" s="6" t="str">
+        <x:v>HKD</x:v>
+      </x:c>
+      <x:c r="M12" s="6" t="str">
+        <x:v>channel: WEB
+schedule: FUTURE</x:v>
+      </x:c>
+      <x:c r="N12" s="6" t="str">
+        <x:v>PAYMENT_POSTCHECK</x:v>
+      </x:c>
+      <x:c r="O12" s="6" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="P12" s="6" t="str">
+        <x:v>expectedStatus: SUCCESS
+expectedRejectCode: '0000'
+effectedRows: 1
+status: POSTED
+Keyword1: PAYMENT
+Keyword2: POSTED</x:v>
+      </x:c>
+      <x:c r="Q12" s="6" t="str">
+        <x:v>Scheduled/future-dated transfer.</x:v>
+      </x:c>
+      <x:c r="R12" s="6" t="str">
+        <x:v>ATT should ignore this</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A13" s="6" t="str">
+        <x:v>TC012</x:v>
+      </x:c>
+      <x:c r="B13" s="6" t="str">
+        <x:v>Recurring transfer first execution success</x:v>
+      </x:c>
+      <x:c r="C13" s="6" t="str">
+        <x:v>regression,recurring</x:v>
+      </x:c>
+      <x:c r="D13" s="6" t="str">
+        <x:v>PAYMENT</x:v>
+      </x:c>
+      <x:c r="E13" s="6" t="str">
+        <x:v>PAYMENT_PRECHECK</x:v>
+      </x:c>
+      <x:c r="F13" s="6" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="G13" s="6" t="str">
+        <x:v>minAccountRows: 1</x:v>
+      </x:c>
+      <x:c r="H13" s="6" t="str">
+        <x:v>PAYMENT_TRANSFER</x:v>
+      </x:c>
+      <x:c r="I13" s="6" t="str">
+        <x:v>811123</x:v>
+      </x:c>
+      <x:c r="J13" s="6" t="str">
+        <x:v>922232</x:v>
+      </x:c>
+      <x:c r="K13" s="6" t="str">
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="L13" s="6" t="str">
+        <x:v>HKD</x:v>
+      </x:c>
+      <x:c r="M13" s="6" t="str">
+        <x:v>channel: MOBILE
+schedule: RECURRING</x:v>
+      </x:c>
+      <x:c r="N13" s="6" t="str">
+        <x:v>PAYMENT_POSTCHECK</x:v>
+      </x:c>
+      <x:c r="O13" s="6" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="P13" s="6" t="str">
+        <x:v>expectedStatus: SUCCESS
+expectedRejectCode: '0000'
+effectedRows: 1
+status: POSTED
+Keyword1: PAYMENT
+Keyword2: POSTED</x:v>
+      </x:c>
+      <x:c r="Q13" s="6" t="str">
+        <x:v>Recurring payment first run.</x:v>
+      </x:c>
+      <x:c r="R13" s="6" t="str">
+        <x:v>ATT should ignore this</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A14" s="6" t="str">
+        <x:v>TC013</x:v>
+      </x:c>
+      <x:c r="B14" s="6" t="str">
+        <x:v>Night batch transfer success</x:v>
+      </x:c>
+      <x:c r="C14" s="6" t="str">
+        <x:v>regression,batch,night</x:v>
+      </x:c>
+      <x:c r="D14" s="6" t="str">
+        <x:v>PAYMENT</x:v>
+      </x:c>
+      <x:c r="E14" s="6" t="str">
+        <x:v>PAYMENT_PRECHECK</x:v>
+      </x:c>
+      <x:c r="F14" s="6" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="G14" s="6" t="str">
+        <x:v>minAccountRows: 1</x:v>
+      </x:c>
+      <x:c r="H14" s="6" t="str">
+        <x:v>PAYMENT_TRANSFER</x:v>
+      </x:c>
+      <x:c r="I14" s="6" t="str">
+        <x:v>811124</x:v>
+      </x:c>
+      <x:c r="J14" s="6" t="str">
+        <x:v>922233</x:v>
+      </x:c>
+      <x:c r="K14" s="6" t="str">
+        <x:v>640</x:v>
+      </x:c>
+      <x:c r="L14" s="6" t="str">
+        <x:v>HKD</x:v>
+      </x:c>
+      <x:c r="M14" s="6" t="str">
+        <x:v>channel: BATCH
+window: NIGHT</x:v>
+      </x:c>
+      <x:c r="N14" s="6" t="str">
+        <x:v>PAYMENT_POSTCHECK</x:v>
+      </x:c>
+      <x:c r="O14" s="6" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="P14" s="6" t="str">
+        <x:v>expectedStatus: SUCCESS
+expectedRejectCode: '0000'
+effectedRows: 1
+status: POSTED
+Keyword1: PAYMENT
+Keyword2: POSTED</x:v>
+      </x:c>
+      <x:c r="Q14" s="6" t="str">
+        <x:v>Night batch processing scenario.</x:v>
+      </x:c>
+      <x:c r="R14" s="6" t="str">
+        <x:v>ATT should ignore this</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A15" s="6" t="str">
+        <x:v>TC014</x:v>
+      </x:c>
+      <x:c r="B15" s="6" t="str">
+        <x:v>Fee-bearing transfer success</x:v>
+      </x:c>
+      <x:c r="C15" s="6" t="str">
+        <x:v>regression,fee</x:v>
+      </x:c>
+      <x:c r="D15" s="6" t="str">
+        <x:v>PAYMENT</x:v>
+      </x:c>
+      <x:c r="E15" s="6" t="str">
+        <x:v>PAYMENT_PRECHECK</x:v>
+      </x:c>
+      <x:c r="F15" s="6" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="G15" s="6" t="str">
+        <x:v>minAccountRows: 1</x:v>
+      </x:c>
+      <x:c r="H15" s="6" t="str">
+        <x:v>PAYMENT_TRANSFER</x:v>
+      </x:c>
+      <x:c r="I15" s="6" t="str">
+        <x:v>811125</x:v>
+      </x:c>
+      <x:c r="J15" s="6" t="str">
+        <x:v>922234</x:v>
+      </x:c>
+      <x:c r="K15" s="6" t="str">
+        <x:v>1280</x:v>
+      </x:c>
+      <x:c r="L15" s="6" t="str">
+        <x:v>HKD</x:v>
+      </x:c>
+      <x:c r="M15" s="6" t="str">
+        <x:v>channel: WEB
+feeMode: SHA</x:v>
+      </x:c>
+      <x:c r="N15" s="6" t="str">
+        <x:v>PAYMENT_POSTCHECK</x:v>
+      </x:c>
+      <x:c r="O15" s="6" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="P15" s="6" t="str">
+        <x:v>expectedStatus: SUCCESS
+expectedRejectCode: '0000'
+effectedRows: 1
+status: POSTED
+Keyword1: PAYMENT
+Keyword2: POSTED</x:v>
+      </x:c>
+      <x:c r="Q15" s="6" t="str">
+        <x:v>Transfer with shared fee mode.</x:v>
+      </x:c>
+      <x:c r="R15" s="6" t="str">
+        <x:v>ATT should ignore this</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A16" s="6" t="str">
+        <x:v>TC015</x:v>
+      </x:c>
+      <x:c r="B16" s="6" t="str">
+        <x:v>No-fee internal transfer success</x:v>
+      </x:c>
+      <x:c r="C16" s="6" t="str">
+        <x:v>regression,no-fee,internal</x:v>
+      </x:c>
+      <x:c r="D16" s="6" t="str">
+        <x:v>PAYMENT</x:v>
+      </x:c>
+      <x:c r="E16" s="6" t="str">
+        <x:v>PAYMENT_PRECHECK</x:v>
+      </x:c>
+      <x:c r="F16" s="6" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="G16" s="6" t="str">
+        <x:v>minAccountRows: 1</x:v>
+      </x:c>
+      <x:c r="H16" s="6" t="str">
+        <x:v>PAYMENT_TRANSFER</x:v>
+      </x:c>
+      <x:c r="I16" s="6" t="str">
+        <x:v>811126</x:v>
+      </x:c>
+      <x:c r="J16" s="6" t="str">
+        <x:v>922235</x:v>
+      </x:c>
+      <x:c r="K16" s="6" t="str">
+        <x:v>1280</x:v>
+      </x:c>
+      <x:c r="L16" s="6" t="str">
+        <x:v>HKD</x:v>
+      </x:c>
+      <x:c r="M16" s="6" t="str">
+        <x:v>channel: WEB
+feeMode: WAIVED</x:v>
+      </x:c>
+      <x:c r="N16" s="6" t="str">
+        <x:v>PAYMENT_POSTCHECK</x:v>
+      </x:c>
+      <x:c r="O16" s="6" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="P16" s="6" t="str">
+        <x:v>expectedStatus: SUCCESS
+expectedRejectCode: '0000'
+effectedRows: 1
+status: POSTED
+Keyword1: PAYMENT
+Keyword2: POSTED</x:v>
+      </x:c>
+      <x:c r="Q16" s="6" t="str">
+        <x:v>Internal no-fee transfer.</x:v>
+      </x:c>
+      <x:c r="R16" s="6" t="str">
+        <x:v>ATT should ignore this</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A17" s="6" t="str">
+        <x:v>TC016</x:v>
+      </x:c>
+      <x:c r="B17" s="6" t="str">
+        <x:v>Decimal cents transfer success</x:v>
+      </x:c>
+      <x:c r="C17" s="6" t="str">
+        <x:v>regression,decimal</x:v>
+      </x:c>
+      <x:c r="D17" s="6" t="str">
+        <x:v>PAYMENT</x:v>
+      </x:c>
+      <x:c r="E17" s="6" t="str">
+        <x:v>PAYMENT_PRECHECK</x:v>
+      </x:c>
+      <x:c r="F17" s="6" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="G17" s="6" t="str">
+        <x:v>minAccountRows: 1</x:v>
+      </x:c>
+      <x:c r="H17" s="6" t="str">
+        <x:v>PAYMENT_TRANSFER</x:v>
+      </x:c>
+      <x:c r="I17" s="6" t="str">
+        <x:v>811127</x:v>
+      </x:c>
+      <x:c r="J17" s="6" t="str">
+        <x:v>922236</x:v>
+      </x:c>
+      <x:c r="K17" s="6" t="str">
+        <x:v>10.01</x:v>
+      </x:c>
+      <x:c r="L17" s="6" t="str">
+        <x:v>HKD</x:v>
+      </x:c>
+      <x:c r="M17" s="6" t="str">
+        <x:v>channel: MOBILE
+precision: CENT</x:v>
+      </x:c>
+      <x:c r="N17" s="6" t="str">
+        <x:v>PAYMENT_POSTCHECK</x:v>
+      </x:c>
+      <x:c r="O17" s="6" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="P17" s="6" t="str">
+        <x:v>expectedStatus: SUCCESS
+expectedRejectCode: '0000'
+effectedRows: 1
+status: POSTED
+Keyword1: PAYMENT
+Keyword2: POSTED</x:v>
+      </x:c>
+      <x:c r="Q17" s="6" t="str">
+        <x:v>Cent precision amount.</x:v>
+      </x:c>
+      <x:c r="R17" s="6" t="str">
+        <x:v>ATT should ignore this</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A18" s="6" t="str">
+        <x:v>TC017</x:v>
+      </x:c>
+      <x:c r="B18" s="6" t="str">
+        <x:v>Maximum daily limit boundary success</x:v>
+      </x:c>
+      <x:c r="C18" s="6" t="str">
+        <x:v>regression,boundary,limit</x:v>
+      </x:c>
+      <x:c r="D18" s="6" t="str">
+        <x:v>PAYMENT</x:v>
+      </x:c>
+      <x:c r="E18" s="6" t="str">
+        <x:v>PAYMENT_PRECHECK</x:v>
+      </x:c>
+      <x:c r="F18" s="6" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="G18" s="6" t="str">
+        <x:v>minAccountRows: 1</x:v>
+      </x:c>
+      <x:c r="H18" s="6" t="str">
+        <x:v>PAYMENT_TRANSFER</x:v>
+      </x:c>
+      <x:c r="I18" s="6" t="str">
+        <x:v>811128</x:v>
+      </x:c>
+      <x:c r="J18" s="6" t="str">
+        <x:v>922237</x:v>
+      </x:c>
+      <x:c r="K18" s="6" t="str">
+        <x:v>1000000</x:v>
+      </x:c>
+      <x:c r="L18" s="6" t="str">
+        <x:v>HKD</x:v>
+      </x:c>
+      <x:c r="M18" s="6" t="str">
+        <x:v>channel: WEB
+limitScenario: DAILY_MAX</x:v>
+      </x:c>
+      <x:c r="N18" s="6" t="str">
+        <x:v>PAYMENT_POSTCHECK</x:v>
+      </x:c>
+      <x:c r="O18" s="6" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="P18" s="6" t="str">
+        <x:v>expectedStatus: SUCCESS
+expectedRejectCode: '0000'
+effectedRows: 1
+status: POSTED
+Keyword1: PAYMENT
+Keyword2: POSTED</x:v>
+      </x:c>
+      <x:c r="Q18" s="6" t="str">
+        <x:v>Daily limit boundary amount.</x:v>
+      </x:c>
+      <x:c r="R18" s="6" t="str">
+        <x:v>ATT should ignore this</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A19" s="6" t="str">
+        <x:v>TC018</x:v>
+      </x:c>
+      <x:c r="B19" s="6" t="str">
+        <x:v>VIP priority transfer success</x:v>
+      </x:c>
+      <x:c r="C19" s="6" t="str">
+        <x:v>regression,vip,priority</x:v>
+      </x:c>
+      <x:c r="D19" s="6" t="str">
+        <x:v>PAYMENT</x:v>
+      </x:c>
+      <x:c r="E19" s="6" t="str">
+        <x:v>PAYMENT_PRECHECK</x:v>
+      </x:c>
+      <x:c r="F19" s="6" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="G19" s="6" t="str">
+        <x:v>minAccountRows: 1</x:v>
+      </x:c>
+      <x:c r="H19" s="6" t="str">
+        <x:v>PAYMENT_TRANSFER</x:v>
+      </x:c>
+      <x:c r="I19" s="6" t="str">
+        <x:v>811129</x:v>
+      </x:c>
+      <x:c r="J19" s="6" t="str">
+        <x:v>922238</x:v>
+      </x:c>
+      <x:c r="K19" s="6" t="str">
+        <x:v>66000</x:v>
+      </x:c>
+      <x:c r="L19" s="6" t="str">
+        <x:v>HKD</x:v>
+      </x:c>
+      <x:c r="M19" s="6" t="str">
+        <x:v>channel: RM
+customerSegment: VIP</x:v>
+      </x:c>
+      <x:c r="N19" s="6" t="str">
+        <x:v>PAYMENT_POSTCHECK</x:v>
+      </x:c>
+      <x:c r="O19" s="6" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="P19" s="6" t="str">
+        <x:v>expectedStatus: SUCCESS
+expectedRejectCode: '0000'
+effectedRows: 1
+status: POSTED
+Keyword1: PAYMENT
+Keyword2: POSTED</x:v>
+      </x:c>
+      <x:c r="Q19" s="6" t="str">
+        <x:v>VIP customer priority path.</x:v>
+      </x:c>
+      <x:c r="R19" s="6" t="str">
+        <x:v>ATT should ignore this</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A20" s="6" t="str">
+        <x:v>TC019</x:v>
+      </x:c>
+      <x:c r="B20" s="6" t="str">
+        <x:v>Dormant-to-active beneficiary transfer success</x:v>
+      </x:c>
+      <x:c r="C20" s="6" t="str">
+        <x:v>regression,beneficiary</x:v>
+      </x:c>
+      <x:c r="D20" s="6" t="str">
+        <x:v>PAYMENT</x:v>
+      </x:c>
+      <x:c r="E20" s="6" t="str">
+        <x:v>PAYMENT_PRECHECK</x:v>
+      </x:c>
+      <x:c r="F20" s="6" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="G20" s="6" t="str">
+        <x:v>minAccountRows: 1</x:v>
+      </x:c>
+      <x:c r="H20" s="6" t="str">
+        <x:v>PAYMENT_TRANSFER</x:v>
+      </x:c>
+      <x:c r="I20" s="6" t="str">
+        <x:v>811130</x:v>
+      </x:c>
+      <x:c r="J20" s="6" t="str">
+        <x:v>922239</x:v>
+      </x:c>
+      <x:c r="K20" s="6" t="str">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="L20" s="6" t="str">
+        <x:v>HKD</x:v>
+      </x:c>
+      <x:c r="M20" s="6" t="str">
+        <x:v>channel: MOBILE
+beneficiaryState: REACTIVATED</x:v>
+      </x:c>
+      <x:c r="N20" s="6" t="str">
+        <x:v>PAYMENT_POSTCHECK</x:v>
+      </x:c>
+      <x:c r="O20" s="6" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="P20" s="6" t="str">
+        <x:v>expectedStatus: SUCCESS
+expectedRejectCode: '0000'
+effectedRows: 1
+status: POSTED
+Keyword1: PAYMENT
+Keyword2: POSTED</x:v>
+      </x:c>
+      <x:c r="Q20" s="6" t="str">
+        <x:v>Reactivated beneficiary scenario.</x:v>
+      </x:c>
+      <x:c r="R20" s="6" t="str">
+        <x:v>ATT should ignore this</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A21" s="6" t="str">
+        <x:v>TC020</x:v>
+      </x:c>
+      <x:c r="B21" s="6" t="str">
+        <x:v>Reference data with special characters success</x:v>
+      </x:c>
+      <x:c r="C21" s="6" t="str">
+        <x:v>regression,special-char</x:v>
+      </x:c>
+      <x:c r="D21" s="6" t="str">
+        <x:v>PAYMENT</x:v>
+      </x:c>
+      <x:c r="E21" s="6" t="str">
+        <x:v>PAYMENT_PRECHECK</x:v>
+      </x:c>
+      <x:c r="F21" s="6" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="G21" s="6" t="str">
+        <x:v>minAccountRows: 1</x:v>
+      </x:c>
+      <x:c r="H21" s="6" t="str">
+        <x:v>PAYMENT_TRANSFER</x:v>
+      </x:c>
+      <x:c r="I21" s="6" t="str">
+        <x:v>811131</x:v>
+      </x:c>
+      <x:c r="J21" s="6" t="str">
+        <x:v>922240</x:v>
+      </x:c>
+      <x:c r="K21" s="6" t="str">
+        <x:v>321.09</x:v>
+      </x:c>
+      <x:c r="L21" s="6" t="str">
+        <x:v>HKD</x:v>
+      </x:c>
+      <x:c r="M21" s="6" t="str">
+        <x:v>channel: WEB
+customerRef: REF-2026/07 A_B</x:v>
+      </x:c>
+      <x:c r="N21" s="6" t="str">
+        <x:v>PAYMENT_POSTCHECK</x:v>
+      </x:c>
+      <x:c r="O21" s="6" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="P21" s="6" t="str">
+        <x:v>expectedStatus: SUCCESS
+expectedRejectCode: '0000'
+effectedRows: 1
+status: POSTED
+Keyword1: PAYMENT
+Keyword2: POSTED</x:v>
+      </x:c>
+      <x:c r="Q21" s="6" t="str">
+        <x:v>Reference includes dash, slash, space, and underscore.</x:v>
+      </x:c>
+      <x:c r="R21" s="6" t="str">
         <x:v>ATT should ignore this</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
feat: implement ATT V1.2 runtime and release package
</commit_message>
<xml_diff>
--- a/testcase/payment_regression.xlsx
+++ b/testcase/payment_regression.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TestCases" sheetId="1" r:id="R1c901ee28e4c420c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Config" sheetId="2" r:id="R2bdb8b288b344200"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="3" r:id="Raf2e949e057f42a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TestCases" sheetId="1" r:id="R4db849b5c8854b01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Config" sheetId="2" r:id="Rb1b742aa7fb64c81"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="3" r:id="R65ed03356333481f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -283,16 +283,16 @@
     <x:col min="2" max="2" width="35.220001220703125" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="22.559999465942383" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="8" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="17.559999465942383" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="20" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="18.889999389648438" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="17.110000610351562" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="10.890000343322754" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="11.4399995803833" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="8.220000267028809" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="7.110000133514404" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="23.889999389648438" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="18.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="16" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="15.890000343322754" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="15.5600004196167" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="10.890000343322754" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="11.4399995803833" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="8.220000267028809" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="7.110000133514404" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="23.889999389648438" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="41.220001220703125" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="17.440000534057617" hidden="0" customWidth="1"/>
     <x:col min="15" max="15" width="20.889999389648438" hidden="0" customWidth="1"/>
     <x:col min="16" max="16" width="21.329999923706055" hidden="0" customWidth="1"/>
     <x:col min="17" max="17" width="41.220001220703125" hidden="0" customWidth="1"/>
@@ -313,49 +313,41 @@
         <x:v>API</x:v>
       </x:c>
       <x:c r="E1" s="5" t="str">
-        <x:v>PreCheck Template</x:v>
+        <x:v>Pre Stage Template</x:v>
       </x:c>
       <x:c r="F1" s="5" t="str">
-        <x:v>Expected PreCheck Result</x:v>
+        <x:v>Main Stage Template</x:v>
       </x:c>
       <x:c r="G1" s="5" t="str">
-        <x:v>Expected PreCheck Data</x:v>
+        <x:v>Post Stage Template</x:v>
       </x:c>
       <x:c r="H1" s="5" t="str">
-        <x:v>Request Template</x:v>
+        <x:v>Debit Account</x:v>
       </x:c>
       <x:c r="I1" s="5" t="str">
-        <x:v>Debit Account</x:v>
+        <x:v>Credit Account</x:v>
       </x:c>
       <x:c r="J1" s="5" t="str">
-        <x:v>Credit Account</x:v>
+        <x:v>Amount</x:v>
       </x:c>
       <x:c r="K1" s="5" t="str">
-        <x:v>Amount</x:v>
+        <x:v>Currency</x:v>
       </x:c>
       <x:c r="L1" s="5" t="str">
-        <x:v>Currency</x:v>
+        <x:v>Case Data</x:v>
       </x:c>
       <x:c r="M1" s="5" t="str">
-        <x:v>Request Data</x:v>
+        <x:v>Remarks</x:v>
       </x:c>
       <x:c r="N1" s="5" t="str">
-        <x:v>PostCheck Template</x:v>
-      </x:c>
-      <x:c r="O1" s="5" t="str">
-        <x:v>Expected PostCheck Result</x:v>
-      </x:c>
-      <x:c r="P1" s="5" t="str">
-        <x:v>Expected PostCheck Data</x:v>
-      </x:c>
-      <x:c r="Q1" s="5" t="str">
-        <x:v>Remarks</x:v>
-      </x:c>
-      <x:c r="R1" s="5" t="str">
         <x:v>Ignored Helper Column</x:v>
       </x:c>
-    </x:row>
-    <x:row r="2" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="O1"/>
+      <x:c r="P1"/>
+      <x:c r="Q1"/>
+      <x:c r="R1"/>
+    </x:row>
+    <x:row r="2" ht="118.80000305175781" hidden="0" customHeight="1">
       <x:c r="A2" s="6" t="str">
         <x:v>TC001</x:v>
       </x:c>
@@ -369,55 +361,49 @@
         <x:v>PAYMENT</x:v>
       </x:c>
       <x:c r="E2" s="6" t="str">
-        <x:v>PAYMENT_PRECHECK</x:v>
+        <x:v>PAYMENT_PREPARE</x:v>
       </x:c>
       <x:c r="F2" s="6" t="str">
-        <x:v>PASS</x:v>
+        <x:v>PAYMENT_INVOKE</x:v>
       </x:c>
       <x:c r="G2" s="6" t="str">
-        <x:v>minAccountRows: 1</x:v>
+        <x:v>PAYMENT_VERIFY</x:v>
       </x:c>
       <x:c r="H2" s="6" t="str">
-        <x:v>PAYMENT_TRANSFER</x:v>
+        <x:v>111111</x:v>
       </x:c>
       <x:c r="I2" s="6" t="str">
-        <x:v>111111</x:v>
+        <x:v>222222</x:v>
       </x:c>
       <x:c r="J2" s="6" t="str">
-        <x:v>222222</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="K2" s="6" t="str">
-        <x:v>100</x:v>
+        <x:v>HKD</x:v>
       </x:c>
       <x:c r="L2" s="6" t="str">
-        <x:v>HKD</x:v>
+        <x:v>channel: ATM
+priority: NORMAL
+expected:
+  status: SUCCESS
+  rejectCode: '0000'
+  effectRows: 1
+  txnStatus: POSTED
+  keyword1: PAYMENT
+  keyword2: POSTED</x:v>
       </x:c>
       <x:c r="M2" s="6" t="str">
-        <x:v>channel: ATM
-priority: NORMAL</x:v>
+        <x:v>Happy path for ATM HKD transfer.</x:v>
       </x:c>
       <x:c r="N2" s="6" t="str">
-        <x:v>PAYMENT_POSTCHECK</x:v>
-      </x:c>
-      <x:c r="O2" s="6" t="str">
-        <x:v>PASS</x:v>
-      </x:c>
-      <x:c r="P2" s="6" t="str">
-        <x:v>expectedStatus: SUCCESS
-expectedRejectCode: '0000'
-effectedRows: 1
-status: POSTED
-Keyword1: PAYMENT
-Keyword2: POSTED</x:v>
-      </x:c>
-      <x:c r="Q2" s="6" t="str">
-        <x:v>Happy path for ATM HKD transfer.</x:v>
-      </x:c>
-      <x:c r="R2" s="6" t="str">
-        <x:v>ATT should ignore this</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="79.19999694824219" hidden="0" customHeight="1">
+        <x:v>ATT should ignore this</x:v>
+      </x:c>
+      <x:c r="O2"/>
+      <x:c r="P2"/>
+      <x:c r="Q2"/>
+      <x:c r="R2"/>
+    </x:row>
+    <x:row r="3" ht="118.80000305175781" hidden="0" customHeight="1">
       <x:c r="A3" s="6" t="str">
         <x:v>TC002</x:v>
       </x:c>
@@ -431,55 +417,49 @@
         <x:v>PAYMENT</x:v>
       </x:c>
       <x:c r="E3" s="6" t="str">
-        <x:v>PAYMENT_PRECHECK</x:v>
+        <x:v>PAYMENT_PREPARE</x:v>
       </x:c>
       <x:c r="F3" s="6" t="str">
-        <x:v>PASS</x:v>
+        <x:v>PAYMENT_INVOKE</x:v>
       </x:c>
       <x:c r="G3" s="6" t="str">
-        <x:v>minAccountRows: 1</x:v>
+        <x:v>PAYMENT_VERIFY</x:v>
       </x:c>
       <x:c r="H3" s="6" t="str">
-        <x:v>PAYMENT_TRANSFER</x:v>
+        <x:v>111112</x:v>
       </x:c>
       <x:c r="I3" s="6" t="str">
-        <x:v>111112</x:v>
+        <x:v>222223</x:v>
       </x:c>
       <x:c r="J3" s="6" t="str">
-        <x:v>222223</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K3" s="6" t="str">
-        <x:v>1</x:v>
+        <x:v>HKD</x:v>
       </x:c>
       <x:c r="L3" s="6" t="str">
-        <x:v>HKD</x:v>
+        <x:v>channel: MOBILE
+priority: NORMAL
+expected:
+  status: SUCCESS
+  rejectCode: '0000'
+  effectRows: 1
+  txnStatus: POSTED
+  keyword1: PAYMENT
+  keyword2: POSTED</x:v>
       </x:c>
       <x:c r="M3" s="6" t="str">
-        <x:v>channel: MOBILE
-priority: NORMAL</x:v>
+        <x:v>Minimum positive amount through mobile channel.</x:v>
       </x:c>
       <x:c r="N3" s="6" t="str">
-        <x:v>PAYMENT_POSTCHECK</x:v>
-      </x:c>
-      <x:c r="O3" s="6" t="str">
-        <x:v>PASS</x:v>
-      </x:c>
-      <x:c r="P3" s="6" t="str">
-        <x:v>expectedStatus: SUCCESS
-expectedRejectCode: '0000'
-effectedRows: 1
-status: POSTED
-Keyword1: PAYMENT
-Keyword2: POSTED</x:v>
-      </x:c>
-      <x:c r="Q3" s="6" t="str">
-        <x:v>Minimum positive amount through mobile channel.</x:v>
-      </x:c>
-      <x:c r="R3" s="6" t="str">
-        <x:v>ATT should ignore this</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="79.19999694824219" hidden="0" customHeight="1">
+        <x:v>ATT should ignore this</x:v>
+      </x:c>
+      <x:c r="O3"/>
+      <x:c r="P3"/>
+      <x:c r="Q3"/>
+      <x:c r="R3"/>
+    </x:row>
+    <x:row r="4" ht="118.80000305175781" hidden="0" customHeight="1">
       <x:c r="A4" s="6" t="str">
         <x:v>TC003</x:v>
       </x:c>
@@ -493,55 +473,49 @@
         <x:v>PAYMENT</x:v>
       </x:c>
       <x:c r="E4" s="6" t="str">
-        <x:v>PAYMENT_PRECHECK</x:v>
+        <x:v>PAYMENT_PREPARE</x:v>
       </x:c>
       <x:c r="F4" s="6" t="str">
-        <x:v>PASS</x:v>
+        <x:v>PAYMENT_INVOKE</x:v>
       </x:c>
       <x:c r="G4" s="6" t="str">
-        <x:v>minAccountRows: 1</x:v>
+        <x:v>PAYMENT_VERIFY</x:v>
       </x:c>
       <x:c r="H4" s="6" t="str">
-        <x:v>PAYMENT_TRANSFER</x:v>
+        <x:v>111113</x:v>
       </x:c>
       <x:c r="I4" s="6" t="str">
-        <x:v>111113</x:v>
+        <x:v>222224</x:v>
       </x:c>
       <x:c r="J4" s="6" t="str">
-        <x:v>222224</x:v>
+        <x:v>999999.99</x:v>
       </x:c>
       <x:c r="K4" s="6" t="str">
-        <x:v>999999.99</x:v>
+        <x:v>HKD</x:v>
       </x:c>
       <x:c r="L4" s="6" t="str">
-        <x:v>HKD</x:v>
+        <x:v>channel: WEB
+priority: HIGH
+expected:
+  status: SUCCESS
+  rejectCode: '0000'
+  effectRows: 1
+  txnStatus: POSTED
+  keyword1: PAYMENT
+  keyword2: POSTED</x:v>
       </x:c>
       <x:c r="M4" s="6" t="str">
-        <x:v>channel: WEB
-priority: HIGH</x:v>
+        <x:v>Large amount with high priority marker.</x:v>
       </x:c>
       <x:c r="N4" s="6" t="str">
-        <x:v>PAYMENT_POSTCHECK</x:v>
-      </x:c>
-      <x:c r="O4" s="6" t="str">
-        <x:v>PASS</x:v>
-      </x:c>
-      <x:c r="P4" s="6" t="str">
-        <x:v>expectedStatus: SUCCESS
-expectedRejectCode: '0000'
-effectedRows: 1
-status: POSTED
-Keyword1: PAYMENT
-Keyword2: POSTED</x:v>
-      </x:c>
-      <x:c r="Q4" s="6" t="str">
-        <x:v>Large amount with high priority marker.</x:v>
-      </x:c>
-      <x:c r="R4" s="6" t="str">
-        <x:v>ATT should ignore this</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="79.19999694824219" hidden="0" customHeight="1">
+        <x:v>ATT should ignore this</x:v>
+      </x:c>
+      <x:c r="O4"/>
+      <x:c r="P4"/>
+      <x:c r="Q4"/>
+      <x:c r="R4"/>
+    </x:row>
+    <x:row r="5" ht="118.80000305175781" hidden="0" customHeight="1">
       <x:c r="A5" s="6" t="str">
         <x:v>TC004</x:v>
       </x:c>
@@ -555,55 +529,49 @@
         <x:v>PAYMENT</x:v>
       </x:c>
       <x:c r="E5" s="6" t="str">
-        <x:v>PAYMENT_PRECHECK</x:v>
+        <x:v>PAYMENT_PREPARE</x:v>
       </x:c>
       <x:c r="F5" s="6" t="str">
-        <x:v>PASS</x:v>
+        <x:v>PAYMENT_INVOKE</x:v>
       </x:c>
       <x:c r="G5" s="6" t="str">
-        <x:v>minAccountRows: 1</x:v>
+        <x:v>PAYMENT_VERIFY</x:v>
       </x:c>
       <x:c r="H5" s="6" t="str">
-        <x:v>PAYMENT_TRANSFER</x:v>
+        <x:v>111114</x:v>
       </x:c>
       <x:c r="I5" s="6" t="str">
-        <x:v>111114</x:v>
+        <x:v>222225</x:v>
       </x:c>
       <x:c r="J5" s="6" t="str">
-        <x:v>222225</x:v>
+        <x:v>5000</x:v>
       </x:c>
       <x:c r="K5" s="6" t="str">
-        <x:v>5000</x:v>
+        <x:v>HKD</x:v>
       </x:c>
       <x:c r="L5" s="6" t="str">
-        <x:v>HKD</x:v>
+        <x:v>channel: BRANCH
+priority: NORMAL
+expected:
+  status: SUCCESS
+  rejectCode: '0000'
+  effectRows: 1
+  txnStatus: POSTED
+  keyword1: PAYMENT
+  keyword2: POSTED</x:v>
       </x:c>
       <x:c r="M5" s="6" t="str">
-        <x:v>channel: BRANCH
-priority: NORMAL</x:v>
+        <x:v>Branch-assisted transfer.</x:v>
       </x:c>
       <x:c r="N5" s="6" t="str">
-        <x:v>PAYMENT_POSTCHECK</x:v>
-      </x:c>
-      <x:c r="O5" s="6" t="str">
-        <x:v>PASS</x:v>
-      </x:c>
-      <x:c r="P5" s="6" t="str">
-        <x:v>expectedStatus: SUCCESS
-expectedRejectCode: '0000'
-effectedRows: 1
-status: POSTED
-Keyword1: PAYMENT
-Keyword2: POSTED</x:v>
-      </x:c>
-      <x:c r="Q5" s="6" t="str">
-        <x:v>Branch-assisted transfer.</x:v>
-      </x:c>
-      <x:c r="R5" s="6" t="str">
-        <x:v>ATT should ignore this</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="79.19999694824219" hidden="0" customHeight="1">
+        <x:v>ATT should ignore this</x:v>
+      </x:c>
+      <x:c r="O5"/>
+      <x:c r="P5"/>
+      <x:c r="Q5"/>
+      <x:c r="R5"/>
+    </x:row>
+    <x:row r="6" ht="118.80000305175781" hidden="0" customHeight="1">
       <x:c r="A6" s="6" t="str">
         <x:v>TC005</x:v>
       </x:c>
@@ -617,55 +585,49 @@
         <x:v>PAYMENT</x:v>
       </x:c>
       <x:c r="E6" s="6" t="str">
-        <x:v>PAYMENT_PRECHECK</x:v>
+        <x:v>PAYMENT_PREPARE</x:v>
       </x:c>
       <x:c r="F6" s="6" t="str">
-        <x:v>PASS</x:v>
+        <x:v>PAYMENT_INVOKE</x:v>
       </x:c>
       <x:c r="G6" s="6" t="str">
-        <x:v>minAccountRows: 1</x:v>
+        <x:v>PAYMENT_VERIFY</x:v>
       </x:c>
       <x:c r="H6" s="6" t="str">
-        <x:v>PAYMENT_TRANSFER</x:v>
+        <x:v>311115</x:v>
       </x:c>
       <x:c r="I6" s="6" t="str">
-        <x:v>311115</x:v>
+        <x:v>422226</x:v>
       </x:c>
       <x:c r="J6" s="6" t="str">
-        <x:v>422226</x:v>
+        <x:v>88888.88</x:v>
       </x:c>
       <x:c r="K6" s="6" t="str">
-        <x:v>88888.88</x:v>
+        <x:v>HKD</x:v>
       </x:c>
       <x:c r="L6" s="6" t="str">
-        <x:v>HKD</x:v>
+        <x:v>channel: HOST
+purpose: PAYROLL
+expected:
+  status: SUCCESS
+  rejectCode: '0000'
+  effectRows: 1
+  txnStatus: POSTED
+  keyword1: PAYMENT
+  keyword2: POSTED</x:v>
       </x:c>
       <x:c r="M6" s="6" t="str">
-        <x:v>channel: HOST
-purpose: PAYROLL</x:v>
+        <x:v>Corporate payroll-like payment.</x:v>
       </x:c>
       <x:c r="N6" s="6" t="str">
-        <x:v>PAYMENT_POSTCHECK</x:v>
-      </x:c>
-      <x:c r="O6" s="6" t="str">
-        <x:v>PASS</x:v>
-      </x:c>
-      <x:c r="P6" s="6" t="str">
-        <x:v>expectedStatus: SUCCESS
-expectedRejectCode: '0000'
-effectedRows: 1
-status: POSTED
-Keyword1: PAYMENT
-Keyword2: POSTED</x:v>
-      </x:c>
-      <x:c r="Q6" s="6" t="str">
-        <x:v>Corporate payroll-like payment.</x:v>
-      </x:c>
-      <x:c r="R6" s="6" t="str">
-        <x:v>ATT should ignore this</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="79.19999694824219" hidden="0" customHeight="1">
+        <x:v>ATT should ignore this</x:v>
+      </x:c>
+      <x:c r="O6"/>
+      <x:c r="P6"/>
+      <x:c r="Q6"/>
+      <x:c r="R6"/>
+    </x:row>
+    <x:row r="7" ht="118.80000305175781" hidden="0" customHeight="1">
       <x:c r="A7" s="6" t="str">
         <x:v>TC006</x:v>
       </x:c>
@@ -679,55 +641,49 @@
         <x:v>PAYMENT</x:v>
       </x:c>
       <x:c r="E7" s="6" t="str">
-        <x:v>PAYMENT_PRECHECK</x:v>
+        <x:v>PAYMENT_PREPARE</x:v>
       </x:c>
       <x:c r="F7" s="6" t="str">
-        <x:v>PASS</x:v>
+        <x:v>PAYMENT_INVOKE</x:v>
       </x:c>
       <x:c r="G7" s="6" t="str">
-        <x:v>minAccountRows: 1</x:v>
+        <x:v>PAYMENT_VERIFY</x:v>
       </x:c>
       <x:c r="H7" s="6" t="str">
-        <x:v>PAYMENT_TRANSFER</x:v>
+        <x:v>511116</x:v>
       </x:c>
       <x:c r="I7" s="6" t="str">
-        <x:v>511116</x:v>
+        <x:v>622227</x:v>
       </x:c>
       <x:c r="J7" s="6" t="str">
-        <x:v>622227</x:v>
+        <x:v>1234.56</x:v>
       </x:c>
       <x:c r="K7" s="6" t="str">
-        <x:v>1234.56</x:v>
+        <x:v>USD</x:v>
       </x:c>
       <x:c r="L7" s="6" t="str">
-        <x:v>USD</x:v>
+        <x:v>channel: WEB
+fxRequired: true
+expected:
+  status: SUCCESS
+  rejectCode: '0000'
+  effectRows: 1
+  txnStatus: POSTED
+  keyword1: PAYMENT
+  keyword2: POSTED</x:v>
       </x:c>
       <x:c r="M7" s="6" t="str">
-        <x:v>channel: WEB
-fxRequired: true</x:v>
+        <x:v>USD transfer with FX flag.</x:v>
       </x:c>
       <x:c r="N7" s="6" t="str">
-        <x:v>PAYMENT_POSTCHECK</x:v>
-      </x:c>
-      <x:c r="O7" s="6" t="str">
-        <x:v>PASS</x:v>
-      </x:c>
-      <x:c r="P7" s="6" t="str">
-        <x:v>expectedStatus: SUCCESS
-expectedRejectCode: '0000'
-effectedRows: 1
-status: POSTED
-Keyword1: PAYMENT
-Keyword2: POSTED</x:v>
-      </x:c>
-      <x:c r="Q7" s="6" t="str">
-        <x:v>USD transfer with FX flag.</x:v>
-      </x:c>
-      <x:c r="R7" s="6" t="str">
-        <x:v>ATT should ignore this</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="79.19999694824219" hidden="0" customHeight="1">
+        <x:v>ATT should ignore this</x:v>
+      </x:c>
+      <x:c r="O7"/>
+      <x:c r="P7"/>
+      <x:c r="Q7"/>
+      <x:c r="R7"/>
+    </x:row>
+    <x:row r="8" ht="118.80000305175781" hidden="0" customHeight="1">
       <x:c r="A8" s="6" t="str">
         <x:v>TC007</x:v>
       </x:c>
@@ -741,55 +697,49 @@
         <x:v>PAYMENT</x:v>
       </x:c>
       <x:c r="E8" s="6" t="str">
-        <x:v>PAYMENT_PRECHECK</x:v>
+        <x:v>PAYMENT_PREPARE</x:v>
       </x:c>
       <x:c r="F8" s="6" t="str">
-        <x:v>PASS</x:v>
+        <x:v>PAYMENT_INVOKE</x:v>
       </x:c>
       <x:c r="G8" s="6" t="str">
-        <x:v>minAccountRows: 1</x:v>
+        <x:v>PAYMENT_VERIFY</x:v>
       </x:c>
       <x:c r="H8" s="6" t="str">
-        <x:v>PAYMENT_TRANSFER</x:v>
+        <x:v>511117</x:v>
       </x:c>
       <x:c r="I8" s="6" t="str">
-        <x:v>511117</x:v>
+        <x:v>622228</x:v>
       </x:c>
       <x:c r="J8" s="6" t="str">
-        <x:v>622228</x:v>
+        <x:v>789.01</x:v>
       </x:c>
       <x:c r="K8" s="6" t="str">
-        <x:v>789.01</x:v>
+        <x:v>EUR</x:v>
       </x:c>
       <x:c r="L8" s="6" t="str">
-        <x:v>EUR</x:v>
+        <x:v>channel: WEB
+fxRequired: true
+expected:
+  status: SUCCESS
+  rejectCode: '0000'
+  effectRows: 1
+  txnStatus: POSTED
+  keyword1: PAYMENT
+  keyword2: POSTED</x:v>
       </x:c>
       <x:c r="M8" s="6" t="str">
-        <x:v>channel: WEB
-fxRequired: true</x:v>
+        <x:v>EUR payment scenario.</x:v>
       </x:c>
       <x:c r="N8" s="6" t="str">
-        <x:v>PAYMENT_POSTCHECK</x:v>
-      </x:c>
-      <x:c r="O8" s="6" t="str">
-        <x:v>PASS</x:v>
-      </x:c>
-      <x:c r="P8" s="6" t="str">
-        <x:v>expectedStatus: SUCCESS
-expectedRejectCode: '0000'
-effectedRows: 1
-status: POSTED
-Keyword1: PAYMENT
-Keyword2: POSTED</x:v>
-      </x:c>
-      <x:c r="Q8" s="6" t="str">
-        <x:v>EUR payment scenario.</x:v>
-      </x:c>
-      <x:c r="R8" s="6" t="str">
-        <x:v>ATT should ignore this</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="79.19999694824219" hidden="0" customHeight="1">
+        <x:v>ATT should ignore this</x:v>
+      </x:c>
+      <x:c r="O8"/>
+      <x:c r="P8"/>
+      <x:c r="Q8"/>
+      <x:c r="R8"/>
+    </x:row>
+    <x:row r="9" ht="118.80000305175781" hidden="0" customHeight="1">
       <x:c r="A9" s="6" t="str">
         <x:v>TC008</x:v>
       </x:c>
@@ -803,55 +753,49 @@
         <x:v>PAYMENT</x:v>
       </x:c>
       <x:c r="E9" s="6" t="str">
-        <x:v>PAYMENT_PRECHECK</x:v>
+        <x:v>PAYMENT_PREPARE</x:v>
       </x:c>
       <x:c r="F9" s="6" t="str">
-        <x:v>PASS</x:v>
+        <x:v>PAYMENT_INVOKE</x:v>
       </x:c>
       <x:c r="G9" s="6" t="str">
-        <x:v>minAccountRows: 1</x:v>
+        <x:v>PAYMENT_VERIFY</x:v>
       </x:c>
       <x:c r="H9" s="6" t="str">
-        <x:v>PAYMENT_TRANSFER</x:v>
+        <x:v>511118</x:v>
       </x:c>
       <x:c r="I9" s="6" t="str">
-        <x:v>511118</x:v>
+        <x:v>622229</x:v>
       </x:c>
       <x:c r="J9" s="6" t="str">
-        <x:v>622229</x:v>
+        <x:v>3000</x:v>
       </x:c>
       <x:c r="K9" s="6" t="str">
-        <x:v>3000</x:v>
+        <x:v>CNY</x:v>
       </x:c>
       <x:c r="L9" s="6" t="str">
-        <x:v>CNY</x:v>
+        <x:v>channel: MOBILE
+crossBorder: true
+expected:
+  status: SUCCESS
+  rejectCode: '0000'
+  effectRows: 1
+  txnStatus: POSTED
+  keyword1: PAYMENT
+  keyword2: POSTED</x:v>
       </x:c>
       <x:c r="M9" s="6" t="str">
-        <x:v>channel: MOBILE
-crossBorder: true</x:v>
+        <x:v>CNY cross-border style payment.</x:v>
       </x:c>
       <x:c r="N9" s="6" t="str">
-        <x:v>PAYMENT_POSTCHECK</x:v>
-      </x:c>
-      <x:c r="O9" s="6" t="str">
-        <x:v>PASS</x:v>
-      </x:c>
-      <x:c r="P9" s="6" t="str">
-        <x:v>expectedStatus: SUCCESS
-expectedRejectCode: '0000'
-effectedRows: 1
-status: POSTED
-Keyword1: PAYMENT
-Keyword2: POSTED</x:v>
-      </x:c>
-      <x:c r="Q9" s="6" t="str">
-        <x:v>CNY cross-border style payment.</x:v>
-      </x:c>
-      <x:c r="R9" s="6" t="str">
-        <x:v>ATT should ignore this</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="79.19999694824219" hidden="0" customHeight="1">
+        <x:v>ATT should ignore this</x:v>
+      </x:c>
+      <x:c r="O9"/>
+      <x:c r="P9"/>
+      <x:c r="Q9"/>
+      <x:c r="R9"/>
+    </x:row>
+    <x:row r="10" ht="118.80000305175781" hidden="0" customHeight="1">
       <x:c r="A10" s="6" t="str">
         <x:v>TC009</x:v>
       </x:c>
@@ -865,55 +809,49 @@
         <x:v>PAYMENT</x:v>
       </x:c>
       <x:c r="E10" s="6" t="str">
-        <x:v>PAYMENT_PRECHECK</x:v>
+        <x:v>PAYMENT_PREPARE</x:v>
       </x:c>
       <x:c r="F10" s="6" t="str">
-        <x:v>PASS</x:v>
+        <x:v>PAYMENT_INVOKE</x:v>
       </x:c>
       <x:c r="G10" s="6" t="str">
-        <x:v>minAccountRows: 1</x:v>
+        <x:v>PAYMENT_VERIFY</x:v>
       </x:c>
       <x:c r="H10" s="6" t="str">
-        <x:v>PAYMENT_TRANSFER</x:v>
+        <x:v>711119</x:v>
       </x:c>
       <x:c r="I10" s="6" t="str">
-        <x:v>711119</x:v>
+        <x:v>711120</x:v>
       </x:c>
       <x:c r="J10" s="6" t="str">
-        <x:v>711120</x:v>
+        <x:v>250</x:v>
       </x:c>
       <x:c r="K10" s="6" t="str">
-        <x:v>250</x:v>
+        <x:v>HKD</x:v>
       </x:c>
       <x:c r="L10" s="6" t="str">
-        <x:v>HKD</x:v>
+        <x:v>channel: MOBILE
+relationship: OWN_ACCOUNT
+expected:
+  status: SUCCESS
+  rejectCode: '0000'
+  effectRows: 1
+  txnStatus: POSTED
+  keyword1: PAYMENT
+  keyword2: POSTED</x:v>
       </x:c>
       <x:c r="M10" s="6" t="str">
-        <x:v>channel: MOBILE
-relationship: OWN_ACCOUNT</x:v>
+        <x:v>Own-account movement.</x:v>
       </x:c>
       <x:c r="N10" s="6" t="str">
-        <x:v>PAYMENT_POSTCHECK</x:v>
-      </x:c>
-      <x:c r="O10" s="6" t="str">
-        <x:v>PASS</x:v>
-      </x:c>
-      <x:c r="P10" s="6" t="str">
-        <x:v>expectedStatus: SUCCESS
-expectedRejectCode: '0000'
-effectedRows: 1
-status: POSTED
-Keyword1: PAYMENT
-Keyword2: POSTED</x:v>
-      </x:c>
-      <x:c r="Q10" s="6" t="str">
-        <x:v>Own-account movement.</x:v>
-      </x:c>
-      <x:c r="R10" s="6" t="str">
-        <x:v>ATT should ignore this</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="79.19999694824219" hidden="0" customHeight="1">
+        <x:v>ATT should ignore this</x:v>
+      </x:c>
+      <x:c r="O10"/>
+      <x:c r="P10"/>
+      <x:c r="Q10"/>
+      <x:c r="R10"/>
+    </x:row>
+    <x:row r="11" ht="118.80000305175781" hidden="0" customHeight="1">
       <x:c r="A11" s="6" t="str">
         <x:v>TC010</x:v>
       </x:c>
@@ -927,55 +865,49 @@
         <x:v>PAYMENT</x:v>
       </x:c>
       <x:c r="E11" s="6" t="str">
-        <x:v>PAYMENT_PRECHECK</x:v>
+        <x:v>PAYMENT_PREPARE</x:v>
       </x:c>
       <x:c r="F11" s="6" t="str">
-        <x:v>PASS</x:v>
+        <x:v>PAYMENT_INVOKE</x:v>
       </x:c>
       <x:c r="G11" s="6" t="str">
-        <x:v>minAccountRows: 1</x:v>
+        <x:v>PAYMENT_VERIFY</x:v>
       </x:c>
       <x:c r="H11" s="6" t="str">
-        <x:v>PAYMENT_TRANSFER</x:v>
+        <x:v>711121</x:v>
       </x:c>
       <x:c r="I11" s="6" t="str">
-        <x:v>711121</x:v>
+        <x:v>822230</x:v>
       </x:c>
       <x:c r="J11" s="6" t="str">
-        <x:v>822230</x:v>
+        <x:v>750</x:v>
       </x:c>
       <x:c r="K11" s="6" t="str">
-        <x:v>750</x:v>
+        <x:v>HKD</x:v>
       </x:c>
       <x:c r="L11" s="6" t="str">
-        <x:v>HKD</x:v>
+        <x:v>channel: WEB
+relationship: THIRD_PARTY
+expected:
+  status: SUCCESS
+  rejectCode: '0000'
+  effectRows: 1
+  txnStatus: POSTED
+  keyword1: PAYMENT
+  keyword2: POSTED</x:v>
       </x:c>
       <x:c r="M11" s="6" t="str">
-        <x:v>channel: WEB
-relationship: THIRD_PARTY</x:v>
+        <x:v>Third-party local transfer.</x:v>
       </x:c>
       <x:c r="N11" s="6" t="str">
-        <x:v>PAYMENT_POSTCHECK</x:v>
-      </x:c>
-      <x:c r="O11" s="6" t="str">
-        <x:v>PASS</x:v>
-      </x:c>
-      <x:c r="P11" s="6" t="str">
-        <x:v>expectedStatus: SUCCESS
-expectedRejectCode: '0000'
-effectedRows: 1
-status: POSTED
-Keyword1: PAYMENT
-Keyword2: POSTED</x:v>
-      </x:c>
-      <x:c r="Q11" s="6" t="str">
-        <x:v>Third-party local transfer.</x:v>
-      </x:c>
-      <x:c r="R11" s="6" t="str">
-        <x:v>ATT should ignore this</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="79.19999694824219" hidden="0" customHeight="1">
+        <x:v>ATT should ignore this</x:v>
+      </x:c>
+      <x:c r="O11"/>
+      <x:c r="P11"/>
+      <x:c r="Q11"/>
+      <x:c r="R11"/>
+    </x:row>
+    <x:row r="12" ht="118.80000305175781" hidden="0" customHeight="1">
       <x:c r="A12" s="6" t="str">
         <x:v>TC011</x:v>
       </x:c>
@@ -989,55 +921,49 @@
         <x:v>PAYMENT</x:v>
       </x:c>
       <x:c r="E12" s="6" t="str">
-        <x:v>PAYMENT_PRECHECK</x:v>
+        <x:v>PAYMENT_PREPARE</x:v>
       </x:c>
       <x:c r="F12" s="6" t="str">
-        <x:v>PASS</x:v>
+        <x:v>PAYMENT_INVOKE</x:v>
       </x:c>
       <x:c r="G12" s="6" t="str">
-        <x:v>minAccountRows: 1</x:v>
+        <x:v>PAYMENT_VERIFY</x:v>
       </x:c>
       <x:c r="H12" s="6" t="str">
-        <x:v>PAYMENT_TRANSFER</x:v>
+        <x:v>811122</x:v>
       </x:c>
       <x:c r="I12" s="6" t="str">
-        <x:v>811122</x:v>
+        <x:v>922231</x:v>
       </x:c>
       <x:c r="J12" s="6" t="str">
-        <x:v>922231</x:v>
+        <x:v>1200</x:v>
       </x:c>
       <x:c r="K12" s="6" t="str">
-        <x:v>1200</x:v>
+        <x:v>HKD</x:v>
       </x:c>
       <x:c r="L12" s="6" t="str">
-        <x:v>HKD</x:v>
+        <x:v>channel: WEB
+schedule: FUTURE
+expected:
+  status: SUCCESS
+  rejectCode: '0000'
+  effectRows: 1
+  txnStatus: POSTED
+  keyword1: PAYMENT
+  keyword2: POSTED</x:v>
       </x:c>
       <x:c r="M12" s="6" t="str">
-        <x:v>channel: WEB
-schedule: FUTURE</x:v>
+        <x:v>Scheduled/future-dated transfer.</x:v>
       </x:c>
       <x:c r="N12" s="6" t="str">
-        <x:v>PAYMENT_POSTCHECK</x:v>
-      </x:c>
-      <x:c r="O12" s="6" t="str">
-        <x:v>PASS</x:v>
-      </x:c>
-      <x:c r="P12" s="6" t="str">
-        <x:v>expectedStatus: SUCCESS
-expectedRejectCode: '0000'
-effectedRows: 1
-status: POSTED
-Keyword1: PAYMENT
-Keyword2: POSTED</x:v>
-      </x:c>
-      <x:c r="Q12" s="6" t="str">
-        <x:v>Scheduled/future-dated transfer.</x:v>
-      </x:c>
-      <x:c r="R12" s="6" t="str">
-        <x:v>ATT should ignore this</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="79.19999694824219" hidden="0" customHeight="1">
+        <x:v>ATT should ignore this</x:v>
+      </x:c>
+      <x:c r="O12"/>
+      <x:c r="P12"/>
+      <x:c r="Q12"/>
+      <x:c r="R12"/>
+    </x:row>
+    <x:row r="13" ht="118.80000305175781" hidden="0" customHeight="1">
       <x:c r="A13" s="6" t="str">
         <x:v>TC012</x:v>
       </x:c>
@@ -1051,55 +977,49 @@
         <x:v>PAYMENT</x:v>
       </x:c>
       <x:c r="E13" s="6" t="str">
-        <x:v>PAYMENT_PRECHECK</x:v>
+        <x:v>PAYMENT_PREPARE</x:v>
       </x:c>
       <x:c r="F13" s="6" t="str">
-        <x:v>PASS</x:v>
+        <x:v>PAYMENT_INVOKE</x:v>
       </x:c>
       <x:c r="G13" s="6" t="str">
-        <x:v>minAccountRows: 1</x:v>
+        <x:v>PAYMENT_VERIFY</x:v>
       </x:c>
       <x:c r="H13" s="6" t="str">
-        <x:v>PAYMENT_TRANSFER</x:v>
+        <x:v>811123</x:v>
       </x:c>
       <x:c r="I13" s="6" t="str">
-        <x:v>811123</x:v>
+        <x:v>922232</x:v>
       </x:c>
       <x:c r="J13" s="6" t="str">
-        <x:v>922232</x:v>
+        <x:v>300</x:v>
       </x:c>
       <x:c r="K13" s="6" t="str">
-        <x:v>300</x:v>
+        <x:v>HKD</x:v>
       </x:c>
       <x:c r="L13" s="6" t="str">
-        <x:v>HKD</x:v>
+        <x:v>channel: MOBILE
+schedule: RECURRING
+expected:
+  status: SUCCESS
+  rejectCode: '0000'
+  effectRows: 1
+  txnStatus: POSTED
+  keyword1: PAYMENT
+  keyword2: POSTED</x:v>
       </x:c>
       <x:c r="M13" s="6" t="str">
-        <x:v>channel: MOBILE
-schedule: RECURRING</x:v>
+        <x:v>Recurring payment first run.</x:v>
       </x:c>
       <x:c r="N13" s="6" t="str">
-        <x:v>PAYMENT_POSTCHECK</x:v>
-      </x:c>
-      <x:c r="O13" s="6" t="str">
-        <x:v>PASS</x:v>
-      </x:c>
-      <x:c r="P13" s="6" t="str">
-        <x:v>expectedStatus: SUCCESS
-expectedRejectCode: '0000'
-effectedRows: 1
-status: POSTED
-Keyword1: PAYMENT
-Keyword2: POSTED</x:v>
-      </x:c>
-      <x:c r="Q13" s="6" t="str">
-        <x:v>Recurring payment first run.</x:v>
-      </x:c>
-      <x:c r="R13" s="6" t="str">
-        <x:v>ATT should ignore this</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="79.19999694824219" hidden="0" customHeight="1">
+        <x:v>ATT should ignore this</x:v>
+      </x:c>
+      <x:c r="O13"/>
+      <x:c r="P13"/>
+      <x:c r="Q13"/>
+      <x:c r="R13"/>
+    </x:row>
+    <x:row r="14" ht="118.80000305175781" hidden="0" customHeight="1">
       <x:c r="A14" s="6" t="str">
         <x:v>TC013</x:v>
       </x:c>
@@ -1113,55 +1033,49 @@
         <x:v>PAYMENT</x:v>
       </x:c>
       <x:c r="E14" s="6" t="str">
-        <x:v>PAYMENT_PRECHECK</x:v>
+        <x:v>PAYMENT_PREPARE</x:v>
       </x:c>
       <x:c r="F14" s="6" t="str">
-        <x:v>PASS</x:v>
+        <x:v>PAYMENT_INVOKE</x:v>
       </x:c>
       <x:c r="G14" s="6" t="str">
-        <x:v>minAccountRows: 1</x:v>
+        <x:v>PAYMENT_VERIFY</x:v>
       </x:c>
       <x:c r="H14" s="6" t="str">
-        <x:v>PAYMENT_TRANSFER</x:v>
+        <x:v>811124</x:v>
       </x:c>
       <x:c r="I14" s="6" t="str">
-        <x:v>811124</x:v>
+        <x:v>922233</x:v>
       </x:c>
       <x:c r="J14" s="6" t="str">
-        <x:v>922233</x:v>
+        <x:v>640</x:v>
       </x:c>
       <x:c r="K14" s="6" t="str">
-        <x:v>640</x:v>
+        <x:v>HKD</x:v>
       </x:c>
       <x:c r="L14" s="6" t="str">
-        <x:v>HKD</x:v>
+        <x:v>channel: BATCH
+window: NIGHT
+expected:
+  status: SUCCESS
+  rejectCode: '0000'
+  effectRows: 1
+  txnStatus: POSTED
+  keyword1: PAYMENT
+  keyword2: POSTED</x:v>
       </x:c>
       <x:c r="M14" s="6" t="str">
-        <x:v>channel: BATCH
-window: NIGHT</x:v>
+        <x:v>Night batch processing scenario.</x:v>
       </x:c>
       <x:c r="N14" s="6" t="str">
-        <x:v>PAYMENT_POSTCHECK</x:v>
-      </x:c>
-      <x:c r="O14" s="6" t="str">
-        <x:v>PASS</x:v>
-      </x:c>
-      <x:c r="P14" s="6" t="str">
-        <x:v>expectedStatus: SUCCESS
-expectedRejectCode: '0000'
-effectedRows: 1
-status: POSTED
-Keyword1: PAYMENT
-Keyword2: POSTED</x:v>
-      </x:c>
-      <x:c r="Q14" s="6" t="str">
-        <x:v>Night batch processing scenario.</x:v>
-      </x:c>
-      <x:c r="R14" s="6" t="str">
-        <x:v>ATT should ignore this</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="79.19999694824219" hidden="0" customHeight="1">
+        <x:v>ATT should ignore this</x:v>
+      </x:c>
+      <x:c r="O14"/>
+      <x:c r="P14"/>
+      <x:c r="Q14"/>
+      <x:c r="R14"/>
+    </x:row>
+    <x:row r="15" ht="118.80000305175781" hidden="0" customHeight="1">
       <x:c r="A15" s="6" t="str">
         <x:v>TC014</x:v>
       </x:c>
@@ -1175,55 +1089,49 @@
         <x:v>PAYMENT</x:v>
       </x:c>
       <x:c r="E15" s="6" t="str">
-        <x:v>PAYMENT_PRECHECK</x:v>
+        <x:v>PAYMENT_PREPARE</x:v>
       </x:c>
       <x:c r="F15" s="6" t="str">
-        <x:v>PASS</x:v>
+        <x:v>PAYMENT_INVOKE</x:v>
       </x:c>
       <x:c r="G15" s="6" t="str">
-        <x:v>minAccountRows: 1</x:v>
+        <x:v>PAYMENT_VERIFY</x:v>
       </x:c>
       <x:c r="H15" s="6" t="str">
-        <x:v>PAYMENT_TRANSFER</x:v>
+        <x:v>811125</x:v>
       </x:c>
       <x:c r="I15" s="6" t="str">
-        <x:v>811125</x:v>
+        <x:v>922234</x:v>
       </x:c>
       <x:c r="J15" s="6" t="str">
-        <x:v>922234</x:v>
+        <x:v>1280</x:v>
       </x:c>
       <x:c r="K15" s="6" t="str">
-        <x:v>1280</x:v>
+        <x:v>HKD</x:v>
       </x:c>
       <x:c r="L15" s="6" t="str">
-        <x:v>HKD</x:v>
+        <x:v>channel: WEB
+feeMode: SHA
+expected:
+  status: SUCCESS
+  rejectCode: '0000'
+  effectRows: 1
+  txnStatus: POSTED
+  keyword1: PAYMENT
+  keyword2: POSTED</x:v>
       </x:c>
       <x:c r="M15" s="6" t="str">
-        <x:v>channel: WEB
-feeMode: SHA</x:v>
+        <x:v>Transfer with shared fee mode.</x:v>
       </x:c>
       <x:c r="N15" s="6" t="str">
-        <x:v>PAYMENT_POSTCHECK</x:v>
-      </x:c>
-      <x:c r="O15" s="6" t="str">
-        <x:v>PASS</x:v>
-      </x:c>
-      <x:c r="P15" s="6" t="str">
-        <x:v>expectedStatus: SUCCESS
-expectedRejectCode: '0000'
-effectedRows: 1
-status: POSTED
-Keyword1: PAYMENT
-Keyword2: POSTED</x:v>
-      </x:c>
-      <x:c r="Q15" s="6" t="str">
-        <x:v>Transfer with shared fee mode.</x:v>
-      </x:c>
-      <x:c r="R15" s="6" t="str">
-        <x:v>ATT should ignore this</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="79.19999694824219" hidden="0" customHeight="1">
+        <x:v>ATT should ignore this</x:v>
+      </x:c>
+      <x:c r="O15"/>
+      <x:c r="P15"/>
+      <x:c r="Q15"/>
+      <x:c r="R15"/>
+    </x:row>
+    <x:row r="16" ht="118.80000305175781" hidden="0" customHeight="1">
       <x:c r="A16" s="6" t="str">
         <x:v>TC015</x:v>
       </x:c>
@@ -1237,55 +1145,49 @@
         <x:v>PAYMENT</x:v>
       </x:c>
       <x:c r="E16" s="6" t="str">
-        <x:v>PAYMENT_PRECHECK</x:v>
+        <x:v>PAYMENT_PREPARE</x:v>
       </x:c>
       <x:c r="F16" s="6" t="str">
-        <x:v>PASS</x:v>
+        <x:v>PAYMENT_INVOKE</x:v>
       </x:c>
       <x:c r="G16" s="6" t="str">
-        <x:v>minAccountRows: 1</x:v>
+        <x:v>PAYMENT_VERIFY</x:v>
       </x:c>
       <x:c r="H16" s="6" t="str">
-        <x:v>PAYMENT_TRANSFER</x:v>
+        <x:v>811126</x:v>
       </x:c>
       <x:c r="I16" s="6" t="str">
-        <x:v>811126</x:v>
+        <x:v>922235</x:v>
       </x:c>
       <x:c r="J16" s="6" t="str">
-        <x:v>922235</x:v>
+        <x:v>1280</x:v>
       </x:c>
       <x:c r="K16" s="6" t="str">
-        <x:v>1280</x:v>
+        <x:v>HKD</x:v>
       </x:c>
       <x:c r="L16" s="6" t="str">
-        <x:v>HKD</x:v>
+        <x:v>channel: WEB
+feeMode: WAIVED
+expected:
+  status: SUCCESS
+  rejectCode: '0000'
+  effectRows: 1
+  txnStatus: POSTED
+  keyword1: PAYMENT
+  keyword2: POSTED</x:v>
       </x:c>
       <x:c r="M16" s="6" t="str">
-        <x:v>channel: WEB
-feeMode: WAIVED</x:v>
+        <x:v>Internal no-fee transfer.</x:v>
       </x:c>
       <x:c r="N16" s="6" t="str">
-        <x:v>PAYMENT_POSTCHECK</x:v>
-      </x:c>
-      <x:c r="O16" s="6" t="str">
-        <x:v>PASS</x:v>
-      </x:c>
-      <x:c r="P16" s="6" t="str">
-        <x:v>expectedStatus: SUCCESS
-expectedRejectCode: '0000'
-effectedRows: 1
-status: POSTED
-Keyword1: PAYMENT
-Keyword2: POSTED</x:v>
-      </x:c>
-      <x:c r="Q16" s="6" t="str">
-        <x:v>Internal no-fee transfer.</x:v>
-      </x:c>
-      <x:c r="R16" s="6" t="str">
-        <x:v>ATT should ignore this</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="79.19999694824219" hidden="0" customHeight="1">
+        <x:v>ATT should ignore this</x:v>
+      </x:c>
+      <x:c r="O16"/>
+      <x:c r="P16"/>
+      <x:c r="Q16"/>
+      <x:c r="R16"/>
+    </x:row>
+    <x:row r="17" ht="118.80000305175781" hidden="0" customHeight="1">
       <x:c r="A17" s="6" t="str">
         <x:v>TC016</x:v>
       </x:c>
@@ -1299,55 +1201,49 @@
         <x:v>PAYMENT</x:v>
       </x:c>
       <x:c r="E17" s="6" t="str">
-        <x:v>PAYMENT_PRECHECK</x:v>
+        <x:v>PAYMENT_PREPARE</x:v>
       </x:c>
       <x:c r="F17" s="6" t="str">
-        <x:v>PASS</x:v>
+        <x:v>PAYMENT_INVOKE</x:v>
       </x:c>
       <x:c r="G17" s="6" t="str">
-        <x:v>minAccountRows: 1</x:v>
+        <x:v>PAYMENT_VERIFY</x:v>
       </x:c>
       <x:c r="H17" s="6" t="str">
-        <x:v>PAYMENT_TRANSFER</x:v>
+        <x:v>811127</x:v>
       </x:c>
       <x:c r="I17" s="6" t="str">
-        <x:v>811127</x:v>
+        <x:v>922236</x:v>
       </x:c>
       <x:c r="J17" s="6" t="str">
-        <x:v>922236</x:v>
+        <x:v>10.01</x:v>
       </x:c>
       <x:c r="K17" s="6" t="str">
-        <x:v>10.01</x:v>
+        <x:v>HKD</x:v>
       </x:c>
       <x:c r="L17" s="6" t="str">
-        <x:v>HKD</x:v>
+        <x:v>channel: MOBILE
+precision: CENT
+expected:
+  status: SUCCESS
+  rejectCode: '0000'
+  effectRows: 1
+  txnStatus: POSTED
+  keyword1: PAYMENT
+  keyword2: POSTED</x:v>
       </x:c>
       <x:c r="M17" s="6" t="str">
-        <x:v>channel: MOBILE
-precision: CENT</x:v>
+        <x:v>Cent precision amount.</x:v>
       </x:c>
       <x:c r="N17" s="6" t="str">
-        <x:v>PAYMENT_POSTCHECK</x:v>
-      </x:c>
-      <x:c r="O17" s="6" t="str">
-        <x:v>PASS</x:v>
-      </x:c>
-      <x:c r="P17" s="6" t="str">
-        <x:v>expectedStatus: SUCCESS
-expectedRejectCode: '0000'
-effectedRows: 1
-status: POSTED
-Keyword1: PAYMENT
-Keyword2: POSTED</x:v>
-      </x:c>
-      <x:c r="Q17" s="6" t="str">
-        <x:v>Cent precision amount.</x:v>
-      </x:c>
-      <x:c r="R17" s="6" t="str">
-        <x:v>ATT should ignore this</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="79.19999694824219" hidden="0" customHeight="1">
+        <x:v>ATT should ignore this</x:v>
+      </x:c>
+      <x:c r="O17"/>
+      <x:c r="P17"/>
+      <x:c r="Q17"/>
+      <x:c r="R17"/>
+    </x:row>
+    <x:row r="18" ht="118.80000305175781" hidden="0" customHeight="1">
       <x:c r="A18" s="6" t="str">
         <x:v>TC017</x:v>
       </x:c>
@@ -1361,55 +1257,49 @@
         <x:v>PAYMENT</x:v>
       </x:c>
       <x:c r="E18" s="6" t="str">
-        <x:v>PAYMENT_PRECHECK</x:v>
+        <x:v>PAYMENT_PREPARE</x:v>
       </x:c>
       <x:c r="F18" s="6" t="str">
-        <x:v>PASS</x:v>
+        <x:v>PAYMENT_INVOKE</x:v>
       </x:c>
       <x:c r="G18" s="6" t="str">
-        <x:v>minAccountRows: 1</x:v>
+        <x:v>PAYMENT_VERIFY</x:v>
       </x:c>
       <x:c r="H18" s="6" t="str">
-        <x:v>PAYMENT_TRANSFER</x:v>
+        <x:v>811128</x:v>
       </x:c>
       <x:c r="I18" s="6" t="str">
-        <x:v>811128</x:v>
+        <x:v>922237</x:v>
       </x:c>
       <x:c r="J18" s="6" t="str">
-        <x:v>922237</x:v>
+        <x:v>1000000</x:v>
       </x:c>
       <x:c r="K18" s="6" t="str">
-        <x:v>1000000</x:v>
+        <x:v>HKD</x:v>
       </x:c>
       <x:c r="L18" s="6" t="str">
-        <x:v>HKD</x:v>
+        <x:v>channel: WEB
+limitScenario: DAILY_MAX
+expected:
+  status: SUCCESS
+  rejectCode: '0000'
+  effectRows: 1
+  txnStatus: POSTED
+  keyword1: PAYMENT
+  keyword2: POSTED</x:v>
       </x:c>
       <x:c r="M18" s="6" t="str">
-        <x:v>channel: WEB
-limitScenario: DAILY_MAX</x:v>
+        <x:v>Daily limit boundary amount.</x:v>
       </x:c>
       <x:c r="N18" s="6" t="str">
-        <x:v>PAYMENT_POSTCHECK</x:v>
-      </x:c>
-      <x:c r="O18" s="6" t="str">
-        <x:v>PASS</x:v>
-      </x:c>
-      <x:c r="P18" s="6" t="str">
-        <x:v>expectedStatus: SUCCESS
-expectedRejectCode: '0000'
-effectedRows: 1
-status: POSTED
-Keyword1: PAYMENT
-Keyword2: POSTED</x:v>
-      </x:c>
-      <x:c r="Q18" s="6" t="str">
-        <x:v>Daily limit boundary amount.</x:v>
-      </x:c>
-      <x:c r="R18" s="6" t="str">
-        <x:v>ATT should ignore this</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="79.19999694824219" hidden="0" customHeight="1">
+        <x:v>ATT should ignore this</x:v>
+      </x:c>
+      <x:c r="O18"/>
+      <x:c r="P18"/>
+      <x:c r="Q18"/>
+      <x:c r="R18"/>
+    </x:row>
+    <x:row r="19" ht="118.80000305175781" hidden="0" customHeight="1">
       <x:c r="A19" s="6" t="str">
         <x:v>TC018</x:v>
       </x:c>
@@ -1423,55 +1313,49 @@
         <x:v>PAYMENT</x:v>
       </x:c>
       <x:c r="E19" s="6" t="str">
-        <x:v>PAYMENT_PRECHECK</x:v>
+        <x:v>PAYMENT_PREPARE</x:v>
       </x:c>
       <x:c r="F19" s="6" t="str">
-        <x:v>PASS</x:v>
+        <x:v>PAYMENT_INVOKE</x:v>
       </x:c>
       <x:c r="G19" s="6" t="str">
-        <x:v>minAccountRows: 1</x:v>
+        <x:v>PAYMENT_VERIFY</x:v>
       </x:c>
       <x:c r="H19" s="6" t="str">
-        <x:v>PAYMENT_TRANSFER</x:v>
+        <x:v>811129</x:v>
       </x:c>
       <x:c r="I19" s="6" t="str">
-        <x:v>811129</x:v>
+        <x:v>922238</x:v>
       </x:c>
       <x:c r="J19" s="6" t="str">
-        <x:v>922238</x:v>
+        <x:v>66000</x:v>
       </x:c>
       <x:c r="K19" s="6" t="str">
-        <x:v>66000</x:v>
+        <x:v>HKD</x:v>
       </x:c>
       <x:c r="L19" s="6" t="str">
-        <x:v>HKD</x:v>
+        <x:v>channel: RM
+customerSegment: VIP
+expected:
+  status: SUCCESS
+  rejectCode: '0000'
+  effectRows: 1
+  txnStatus: POSTED
+  keyword1: PAYMENT
+  keyword2: POSTED</x:v>
       </x:c>
       <x:c r="M19" s="6" t="str">
-        <x:v>channel: RM
-customerSegment: VIP</x:v>
+        <x:v>VIP customer priority path.</x:v>
       </x:c>
       <x:c r="N19" s="6" t="str">
-        <x:v>PAYMENT_POSTCHECK</x:v>
-      </x:c>
-      <x:c r="O19" s="6" t="str">
-        <x:v>PASS</x:v>
-      </x:c>
-      <x:c r="P19" s="6" t="str">
-        <x:v>expectedStatus: SUCCESS
-expectedRejectCode: '0000'
-effectedRows: 1
-status: POSTED
-Keyword1: PAYMENT
-Keyword2: POSTED</x:v>
-      </x:c>
-      <x:c r="Q19" s="6" t="str">
-        <x:v>VIP customer priority path.</x:v>
-      </x:c>
-      <x:c r="R19" s="6" t="str">
-        <x:v>ATT should ignore this</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" ht="79.19999694824219" hidden="0" customHeight="1">
+        <x:v>ATT should ignore this</x:v>
+      </x:c>
+      <x:c r="O19"/>
+      <x:c r="P19"/>
+      <x:c r="Q19"/>
+      <x:c r="R19"/>
+    </x:row>
+    <x:row r="20" ht="118.80000305175781" hidden="0" customHeight="1">
       <x:c r="A20" s="6" t="str">
         <x:v>TC019</x:v>
       </x:c>
@@ -1485,55 +1369,49 @@
         <x:v>PAYMENT</x:v>
       </x:c>
       <x:c r="E20" s="6" t="str">
-        <x:v>PAYMENT_PRECHECK</x:v>
+        <x:v>PAYMENT_PREPARE</x:v>
       </x:c>
       <x:c r="F20" s="6" t="str">
-        <x:v>PASS</x:v>
+        <x:v>PAYMENT_INVOKE</x:v>
       </x:c>
       <x:c r="G20" s="6" t="str">
-        <x:v>minAccountRows: 1</x:v>
+        <x:v>PAYMENT_VERIFY</x:v>
       </x:c>
       <x:c r="H20" s="6" t="str">
-        <x:v>PAYMENT_TRANSFER</x:v>
+        <x:v>811130</x:v>
       </x:c>
       <x:c r="I20" s="6" t="str">
-        <x:v>811130</x:v>
+        <x:v>922239</x:v>
       </x:c>
       <x:c r="J20" s="6" t="str">
-        <x:v>922239</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="K20" s="6" t="str">
-        <x:v>90</x:v>
+        <x:v>HKD</x:v>
       </x:c>
       <x:c r="L20" s="6" t="str">
-        <x:v>HKD</x:v>
+        <x:v>channel: MOBILE
+beneficiaryState: REACTIVATED
+expected:
+  status: SUCCESS
+  rejectCode: '0000'
+  effectRows: 1
+  txnStatus: POSTED
+  keyword1: PAYMENT
+  keyword2: POSTED</x:v>
       </x:c>
       <x:c r="M20" s="6" t="str">
-        <x:v>channel: MOBILE
-beneficiaryState: REACTIVATED</x:v>
+        <x:v>Reactivated beneficiary scenario.</x:v>
       </x:c>
       <x:c r="N20" s="6" t="str">
-        <x:v>PAYMENT_POSTCHECK</x:v>
-      </x:c>
-      <x:c r="O20" s="6" t="str">
-        <x:v>PASS</x:v>
-      </x:c>
-      <x:c r="P20" s="6" t="str">
-        <x:v>expectedStatus: SUCCESS
-expectedRejectCode: '0000'
-effectedRows: 1
-status: POSTED
-Keyword1: PAYMENT
-Keyword2: POSTED</x:v>
-      </x:c>
-      <x:c r="Q20" s="6" t="str">
-        <x:v>Reactivated beneficiary scenario.</x:v>
-      </x:c>
-      <x:c r="R20" s="6" t="str">
-        <x:v>ATT should ignore this</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" ht="79.19999694824219" hidden="0" customHeight="1">
+        <x:v>ATT should ignore this</x:v>
+      </x:c>
+      <x:c r="O20"/>
+      <x:c r="P20"/>
+      <x:c r="Q20"/>
+      <x:c r="R20"/>
+    </x:row>
+    <x:row r="21" ht="118.80000305175781" hidden="0" customHeight="1">
       <x:c r="A21" s="6" t="str">
         <x:v>TC020</x:v>
       </x:c>
@@ -1547,53 +1425,47 @@
         <x:v>PAYMENT</x:v>
       </x:c>
       <x:c r="E21" s="6" t="str">
-        <x:v>PAYMENT_PRECHECK</x:v>
+        <x:v>PAYMENT_PREPARE</x:v>
       </x:c>
       <x:c r="F21" s="6" t="str">
-        <x:v>PASS</x:v>
+        <x:v>PAYMENT_INVOKE</x:v>
       </x:c>
       <x:c r="G21" s="6" t="str">
-        <x:v>minAccountRows: 1</x:v>
+        <x:v>PAYMENT_VERIFY</x:v>
       </x:c>
       <x:c r="H21" s="6" t="str">
-        <x:v>PAYMENT_TRANSFER</x:v>
+        <x:v>811131</x:v>
       </x:c>
       <x:c r="I21" s="6" t="str">
-        <x:v>811131</x:v>
+        <x:v>922240</x:v>
       </x:c>
       <x:c r="J21" s="6" t="str">
-        <x:v>922240</x:v>
+        <x:v>321.09</x:v>
       </x:c>
       <x:c r="K21" s="6" t="str">
-        <x:v>321.09</x:v>
+        <x:v>HKD</x:v>
       </x:c>
       <x:c r="L21" s="6" t="str">
-        <x:v>HKD</x:v>
+        <x:v>channel: WEB
+customerRef: REF-2026/07 A_B
+expected:
+  status: SUCCESS
+  rejectCode: '0000'
+  effectRows: 1
+  txnStatus: POSTED
+  keyword1: PAYMENT
+  keyword2: POSTED</x:v>
       </x:c>
       <x:c r="M21" s="6" t="str">
-        <x:v>channel: WEB
-customerRef: REF-2026/07 A_B</x:v>
+        <x:v>Reference includes dash, slash, space, and underscore.</x:v>
       </x:c>
       <x:c r="N21" s="6" t="str">
-        <x:v>PAYMENT_POSTCHECK</x:v>
-      </x:c>
-      <x:c r="O21" s="6" t="str">
-        <x:v>PASS</x:v>
-      </x:c>
-      <x:c r="P21" s="6" t="str">
-        <x:v>expectedStatus: SUCCESS
-expectedRejectCode: '0000'
-effectedRows: 1
-status: POSTED
-Keyword1: PAYMENT
-Keyword2: POSTED</x:v>
-      </x:c>
-      <x:c r="Q21" s="6" t="str">
-        <x:v>Reference includes dash, slash, space, and underscore.</x:v>
-      </x:c>
-      <x:c r="R21" s="6" t="str">
-        <x:v>ATT should ignore this</x:v>
-      </x:c>
+        <x:v>ATT should ignore this</x:v>
+      </x:c>
+      <x:c r="O21"/>
+      <x:c r="P21"/>
+      <x:c r="Q21"/>
+      <x:c r="R21"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>